<commit_message>
Free Friday P1 for assembly without clashing Lis's ECE cover
Move Nikki's LA1 cover to Fri P6 (Katie teaches P5); Fiona's T9 covered
by relief at Fri P6. Resolves the Lis Lowndes Friday P5 double-booking.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Tapping_S2_Specialist_Timetable.xlsx
+++ b/Tapping_S2_Specialist_Timetable.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4434" uniqueCount="445">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4434" uniqueCount="446">
   <si>
     <t>Semester 2 Specialist Timetable (Years 1-6) · colour-coded by specialist</t>
   </si>
@@ -2577,8 +2577,8 @@
 PE</t>
   </si>
   <si>
-    <t xml:space="preserve">Cover T9
-(Dyer)</t>
+    <t xml:space="preserve">Cover LA1
+(Luca)</t>
   </si>
   <si>
     <t>Natalie Carter  ·  specialist (0.6; works Mon/Tue/Wed)</t>
@@ -2976,6 +2976,10 @@
 (class)</t>
   </si>
   <si>
+    <t xml:space="preserve">teacher
+(class)</t>
+  </si>
+  <si>
     <t>T10  ·  Kindy (Donna Campbell)</t>
   </si>
   <si>
@@ -3396,7 +3400,7 @@
     <t>| Caroline Parkin | PP | LA2 | 1 | 320m | 310m | -10m |</t>
   </si>
   <si>
-    <t>| Katie Digney | PP | LA1 | 0.8 | 256m | 250m | -6m |</t>
+    <t>| Katie Digney | PP | LA1 | 0.8 | 256m | 265m | +9m |</t>
   </si>
   <si>
     <t>| Nikki Luca | PP | LA1 | 0.4 | 128m | 105m | -23m |</t>
@@ -14438,8 +14442,8 @@
       <c r="E35" s="20" t="s">
         <v>169</v>
       </c>
-      <c r="F35" s="21" t="s">
-        <v>168</v>
+      <c r="F35" s="9" t="s">
+        <v>268</v>
       </c>
     </row>
     <row r="36" ht="14" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -14470,8 +14474,8 @@
       <c r="E37" s="20" t="s">
         <v>169</v>
       </c>
-      <c r="F37" s="9" t="s">
-        <v>268</v>
+      <c r="F37" s="21" t="s">
+        <v>168</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
@@ -15602,8 +15606,8 @@
       <c r="E107" s="9" t="s">
         <v>284</v>
       </c>
-      <c r="F107" s="22" t="s">
-        <v>285</v>
+      <c r="F107" s="9" t="s">
+        <v>283</v>
       </c>
     </row>
     <row r="108" ht="14" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -15634,8 +15638,8 @@
       <c r="E109" s="9" t="s">
         <v>284</v>
       </c>
-      <c r="F109" s="9" t="s">
-        <v>283</v>
+      <c r="F109" s="22" t="s">
+        <v>285</v>
       </c>
     </row>
     <row r="111" spans="1:6" x14ac:dyDescent="0.25">
@@ -16605,12 +16609,12 @@
         <v>297</v>
       </c>
       <c r="F169" s="22" t="s">
-        <v>285</v>
+        <v>298</v>
       </c>
     </row>
     <row r="171" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A171" s="7" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="B171" s="7"/>
       <c r="C171" s="7"/>
@@ -16867,7 +16871,7 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="23" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="B1" s="23"/>
       <c r="C1" s="23"/>
@@ -17421,8 +17425,8 @@
       <c r="E35" s="20" t="s">
         <v>169</v>
       </c>
-      <c r="F35" s="21" t="s">
-        <v>168</v>
+      <c r="F35" s="9" t="s">
+        <v>268</v>
       </c>
     </row>
     <row r="36" ht="14" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -17453,8 +17457,8 @@
       <c r="E37" s="20" t="s">
         <v>169</v>
       </c>
-      <c r="F37" s="9" t="s">
-        <v>268</v>
+      <c r="F37" s="21" t="s">
+        <v>168</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
@@ -18585,8 +18589,8 @@
       <c r="E107" s="9" t="s">
         <v>284</v>
       </c>
-      <c r="F107" s="22" t="s">
-        <v>285</v>
+      <c r="F107" s="9" t="s">
+        <v>283</v>
       </c>
     </row>
     <row r="108" ht="14" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -18617,8 +18621,8 @@
       <c r="E109" s="9" t="s">
         <v>284</v>
       </c>
-      <c r="F109" s="9" t="s">
-        <v>283</v>
+      <c r="F109" s="22" t="s">
+        <v>285</v>
       </c>
     </row>
     <row r="111" spans="1:6" x14ac:dyDescent="0.25">
@@ -19588,12 +19592,12 @@
         <v>297</v>
       </c>
       <c r="F169" s="22" t="s">
-        <v>285</v>
+        <v>298</v>
       </c>
     </row>
     <row r="171" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A171" s="7" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="B171" s="7"/>
       <c r="C171" s="7"/>
@@ -19849,842 +19853,842 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="23" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" s="24" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" s="24" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" s="24" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" s="24" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" s="24" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" s="24" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" s="24" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" s="24" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" s="24" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" s="23" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" s="24" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" s="24" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" s="24" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" s="24" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" s="24" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" s="24" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" s="24" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26" s="24" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" s="24" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" s="24" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" s="24" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A30" s="24" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A31" s="24" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A32" s="24" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" s="24" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A34" s="24" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A35" s="24" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A36" s="24" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A37" s="24" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A40" s="23" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A42" s="24" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A43" s="24" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A44" s="24" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A45" s="24" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A46" s="24" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A47" s="24" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A50" s="23" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A54" s="23" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
     </row>
     <row r="55" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
     </row>
     <row r="56" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
     </row>
     <row r="57" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A57" s="24" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
     </row>
     <row r="58" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A58" s="24" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
     </row>
     <row r="59" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A59" s="24" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
     </row>
     <row r="60" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A60" s="24" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
     </row>
     <row r="61" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A61" s="24" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
     </row>
     <row r="62" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A62" s="24" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
     </row>
     <row r="63" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A63" s="24" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
     </row>
     <row r="64" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A64" s="24" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
     </row>
     <row r="65" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A65" s="24" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
     </row>
     <row r="66" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
     </row>
     <row r="67" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A67" s="24" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
     </row>
     <row r="68" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A68" s="24" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
     </row>
     <row r="69" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A69" s="24" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
     </row>
     <row r="70" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A70" s="24" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
     </row>
     <row r="71" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A71" s="24" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
     </row>
     <row r="72" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A72" s="24" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
     </row>
     <row r="73" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A73" s="24" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
     </row>
     <row r="74" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A74" s="24" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
     </row>
     <row r="75" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A75" s="24" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
     </row>
     <row r="76" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A76" s="24" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
     </row>
     <row r="77" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A77" s="24" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
     </row>
     <row r="78" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A78" s="24" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
     </row>
     <row r="79" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A79" s="24" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
     </row>
     <row r="80" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A80" s="24" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
     </row>
     <row r="81" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A81" s="24" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
     </row>
     <row r="82" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A82" s="24" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
     </row>
     <row r="83" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A83" s="24" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
     </row>
     <row r="84" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
     </row>
     <row r="85" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
     </row>
     <row r="86" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A86" s="23" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
     </row>
     <row r="87" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
     </row>
     <row r="88" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A88" s="24" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
     </row>
     <row r="89" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A89" s="24" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
     </row>
     <row r="90" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A90" s="24" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
     </row>
     <row r="91" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A91" s="24" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
     </row>
     <row r="92" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A92" s="24" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
     </row>
     <row r="93" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A93" s="24" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
     </row>
     <row r="94" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A94" s="24" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
     </row>
     <row r="95" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A95" s="24" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
     </row>
     <row r="96" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A96" s="24" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
     </row>
     <row r="97" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
     </row>
     <row r="98" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
     </row>
     <row r="99" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A99" s="23" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
     </row>
     <row r="100" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
     </row>
     <row r="101" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A101" s="24" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
     </row>
     <row r="102" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A102" s="24" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
     </row>
     <row r="103" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A103" s="24" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
     </row>
     <row r="104" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A104" s="24" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
     </row>
     <row r="105" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A105" s="24" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
     </row>
     <row r="106" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A106" s="24" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
     </row>
     <row r="107" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A107" s="24" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
     </row>
     <row r="108" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A108" s="24" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
     </row>
     <row r="109" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A109" s="24" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
     </row>
     <row r="110" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A110" s="24" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
     </row>
     <row r="111" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A111" s="24" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
     </row>
     <row r="112" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A112" s="24" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
     </row>
     <row r="113" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A113" s="24" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
     </row>
     <row r="114" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A114" s="24" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
     </row>
     <row r="115" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A115" s="24" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
     </row>
     <row r="116" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A116" s="24" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
     </row>
     <row r="117" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A117" s="24" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
     </row>
     <row r="118" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
     </row>
     <row r="119" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
     </row>
     <row r="120" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A120" s="23" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
     </row>
     <row r="121" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
     </row>
     <row r="122" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
     </row>
     <row r="123" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A123" s="24" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
     </row>
     <row r="124" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A124" s="24" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
     </row>
     <row r="125" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A125" s="24" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="126" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A126" s="24" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
     </row>
     <row r="127" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A127" s="24" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
     </row>
     <row r="128" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A128" s="24" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
     </row>
     <row r="129" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A129" s="24" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
     </row>
     <row r="130" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A130" s="24" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
     </row>
     <row r="131" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A131" s="24" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
     </row>
     <row r="132" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A132" s="24" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
     </row>
     <row r="133" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A133" s="24" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
     </row>
     <row r="134" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A134" s="24" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
     </row>
     <row r="135" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A135" s="24" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
     </row>
     <row r="136" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A136" s="24" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
     </row>
     <row r="137" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A137" s="24" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
     </row>
     <row r="138" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A138" s="24" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
     </row>
     <row r="139" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A139" s="24" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
     </row>
     <row r="140" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
     </row>
     <row r="141" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
     </row>
     <row r="142" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A142" s="23" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
     </row>
     <row r="143" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
     </row>
     <row r="144" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
     </row>
     <row r="145" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A145" s="24" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
     </row>
     <row r="146" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A146" s="24" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
     </row>
     <row r="147" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A147" s="24" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
     </row>
     <row r="148" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A148" s="24" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
     </row>
     <row r="149" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A149" s="24" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
     </row>
     <row r="150" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A150" s="24" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
     </row>
     <row r="151" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A151" s="24" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
     </row>
     <row r="152" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
     </row>
     <row r="153" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
     </row>
     <row r="154" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
     </row>
     <row r="155" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A155" s="23" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
     </row>
     <row r="156" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
     </row>
     <row r="157" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
     </row>
     <row r="158" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A158" s="24" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
     </row>
     <row r="159" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A159" s="24" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
     </row>
     <row r="160" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A160" s="24" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
     </row>
     <row r="161" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A161" s="24" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
     </row>
     <row r="162" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A162" s="24" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
     </row>
     <row r="163" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A163" s="24" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
     </row>
     <row r="164" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A164" s="24" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
     </row>
     <row r="165" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A165" s="24" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
     </row>
     <row r="166" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A166" s="24" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
     </row>
     <row r="167" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A167" s="24" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
     </row>
     <row r="168" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
DOTT equity: give Webb (LA22) a Period 6 STEM; trim Lis surplus
LA22 STEM -> Mon P5-6, LA23 STEM -> Tue P3-4, LA23 Visual Art -> Mon P1.
Webb 330->345 (level with other grads); Lis +95->+80; Bell unchanged.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Tapping_S2_Specialist_Timetable.xlsx
+++ b/Tapping_S2_Specialist_Timetable.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4434" uniqueCount="446">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4435" uniqueCount="447">
   <si>
     <t>Semester 2 Specialist Timetable (Years 1-6) · colour-coded by specialist</t>
   </si>
@@ -91,6 +91,23 @@
       </rPr>
       <t xml:space="preserve">  Lis Lowndes</t>
     </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF29A39A"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA17 STEM</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF29A39A"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Chantel Uhe</t>
+    </r>
     <r>
       <rPr>
         <sz val="6"/>
@@ -104,7 +121,7 @@
         <color rgb="FFD98A3D"/>
         <sz val="10"/>
       </rPr>
-      <t>LA23 Visual Art</t>
+      <t>LA21 Visual Art</t>
     </r>
     <r>
       <rPr>
@@ -112,6 +129,88 @@
         <sz val="9"/>
       </rPr>
       <t xml:space="preserve">  Natalie Carter</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF7E57C2"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA6 Auslan</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF7E57C2"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Rachel Walker</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FFD4538A"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA9 Performing Arts</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FFD4538A"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Cheryl Peak</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">P2
+9:40-10:25</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FFD98A3D"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA6 Visual Art</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FFD98A3D"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Natalie Carter</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF1F8A82"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA20 STEM</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF1F8A82"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Lis Lowndes</t>
     </r>
   </si>
   <si>
@@ -121,7 +220,7 @@
         <color rgb="FF29A39A"/>
         <sz val="10"/>
       </rPr>
-      <t>LA17 STEM</t>
+      <t>LA8 STEM</t>
     </r>
     <r>
       <rPr>
@@ -129,6 +228,28 @@
         <sz val="9"/>
       </rPr>
       <t xml:space="preserve">  Chantel Uhe</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF1F8A82"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA24 STEM</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF1F8A82"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Lis Lowndes</t>
     </r>
     <r>
       <rPr>
@@ -143,7 +264,7 @@
         <color rgb="FFD98A3D"/>
         <sz val="10"/>
       </rPr>
-      <t>LA21 Visual Art</t>
+      <t>LA19 Visual Art</t>
     </r>
     <r>
       <rPr>
@@ -152,15 +273,142 @@
       </rPr>
       <t xml:space="preserve">  Natalie Carter</t>
     </r>
-  </si>
-  <si>
+    <r>
+      <rPr>
+        <sz val="6"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FFD4538A"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA20 Performing Arts</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FFD4538A"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Cheryl Peak</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF29A39A"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA17 STEM</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF29A39A"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Chantel Uhe</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF1F8A82"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA14 STEM</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF1F8A82"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Lis Lowndes</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF1F8A82"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA6 PE</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF1F8A82"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Lis Lowndes</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF4A90D9"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA8 PE</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF4A90D9"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Aaron Bell</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF6AA9E0"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA9 PE</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF6AA9E0"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Jake Pevitt</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
     <r>
       <rPr>
         <b/>
         <color rgb="FF7E57C2"/>
         <sz val="10"/>
       </rPr>
-      <t>LA6 Auslan</t>
+      <t>LA14 Auslan</t>
     </r>
     <r>
       <rPr>
@@ -182,7 +430,7 @@
         <color rgb="FFD4538A"/>
         <sz val="10"/>
       </rPr>
-      <t>LA9 Performing Arts</t>
+      <t>LA21 Performing Arts</t>
     </r>
     <r>
       <rPr>
@@ -193,17 +441,161 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">P2
-9:40-10:25</t>
-  </si>
-  <si>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FFD4538A"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA18 Auslan</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FFD4538A"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Cheryl Peak</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF1F8A82"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA15 STEM</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF1F8A82"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Lis Lowndes</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF4A90D9"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA21 Health</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF4A90D9"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Aaron Bell</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">P3
+10:25-11:10</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF1F8A82"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA20 STEM</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF1F8A82"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Lis Lowndes</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF29A39A"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA9 STEM</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF29A39A"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Chantel Uhe</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FFD4538A"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA16 Performing Arts</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FFD4538A"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Cheryl Peak</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF1F8A82"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA23 STEM</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF1F8A82"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Lis Lowndes</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
     <r>
       <rPr>
         <b/>
         <color rgb="FFD98A3D"/>
         <sz val="10"/>
       </rPr>
-      <t>LA6 Visual Art</t>
+      <t>LA14 Visual Art</t>
     </r>
     <r>
       <rPr>
@@ -211,6 +603,67 @@
         <sz val="9"/>
       </rPr>
       <t xml:space="preserve">  Natalie Carter</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF29A39A"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA16 STEM</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF29A39A"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Chantel Uhe</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FFD4538A"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA6 Performing Arts</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FFD4538A"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Cheryl Peak</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF7E57C2"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA8 Auslan</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF7E57C2"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Rachel Walker</t>
     </r>
     <r>
       <rPr>
@@ -225,7 +678,7 @@
         <color rgb="FF1F8A82"/>
         <sz val="10"/>
       </rPr>
-      <t>LA20 STEM</t>
+      <t>LA14 STEM</t>
     </r>
     <r>
       <rPr>
@@ -233,6 +686,222 @@
         <sz val="9"/>
       </rPr>
       <t xml:space="preserve">  Lis Lowndes</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FFD98A3D"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA15 Visual Art</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FFD98A3D"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Natalie Carter</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF1F8A82"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA7 PE</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF1F8A82"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Lis Lowndes</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF4A90D9"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA16 PE</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF4A90D9"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Aaron Bell</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF6AA9E0"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA17 PE</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF6AA9E0"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Jake Pevitt</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF7E57C2"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA15 Auslan</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF7E57C2"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Rachel Walker</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FFD4538A"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA22 Performing Arts</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FFD4538A"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Cheryl Peak</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FFD4538A"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA20 Auslan</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FFD4538A"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Cheryl Peak</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF4A90D9"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA18 Health</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF4A90D9"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Aaron Bell</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF1F8A82"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA15 STEM</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF1F8A82"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Lis Lowndes</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Lunch
+11:10-11:50</t>
+  </si>
+  <si>
+    <t>Lunch (11:10-11:50)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P4
+11:50-12:35</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FFD98A3D"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA18 Visual Art</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FFD98A3D"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Natalie Carter</t>
     </r>
   </si>
   <si>
@@ -242,7 +911,7 @@
         <color rgb="FF29A39A"/>
         <sz val="10"/>
       </rPr>
-      <t>LA8 STEM</t>
+      <t>LA9 STEM</t>
     </r>
     <r>
       <rPr>
@@ -250,6 +919,28 @@
         <sz val="9"/>
       </rPr>
       <t xml:space="preserve">  Chantel Uhe</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FFD4538A"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA17 Performing Arts</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FFD4538A"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Cheryl Peak</t>
     </r>
     <r>
       <rPr>
@@ -264,7 +955,7 @@
         <color rgb="FF1F8A82"/>
         <sz val="10"/>
       </rPr>
-      <t>LA24 STEM</t>
+      <t>LA23 STEM</t>
     </r>
     <r>
       <rPr>
@@ -286,7 +977,46 @@
         <color rgb="FFD98A3D"/>
         <sz val="10"/>
       </rPr>
-      <t>LA19 Visual Art</t>
+      <t>LA7 Visual Art</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FFD98A3D"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Natalie Carter</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF29A39A"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA16 STEM</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF29A39A"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Chantel Uhe</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FFD98A3D"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA22 Visual Art</t>
     </r>
     <r>
       <rPr>
@@ -308,7 +1038,7 @@
         <color rgb="FFD4538A"/>
         <sz val="10"/>
       </rPr>
-      <t>LA20 Performing Arts</t>
+      <t>LA23 Performing Arts</t>
     </r>
     <r>
       <rPr>
@@ -316,6 +1046,259 @@
         <sz val="9"/>
       </rPr>
       <t xml:space="preserve">  Cheryl Peak</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF7E57C2"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA24 Auslan</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF7E57C2"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Rachel Walker</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF1F8A82"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA19 STEM</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF1F8A82"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Lis Lowndes</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF1F8A82"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA14 PE</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF1F8A82"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Lis Lowndes</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF4A90D9"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA15 PE</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF4A90D9"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Aaron Bell</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF6AA9E0"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA21 PE</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF6AA9E0"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Jake Pevitt</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF7E57C2"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA17 Auslan</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF7E57C2"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Rachel Walker</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FFD4538A"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA19 Performing Arts</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FFD4538A"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Cheryl Peak</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FFD4538A"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA23 Auslan</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FFD4538A"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Cheryl Peak</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF4A90D9"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA22 Health</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF4A90D9"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Aaron Bell</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF1F8A82"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA21 STEM</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF1F8A82"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Lis Lowndes</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">P5
+12:35-1:20</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF1F8A82"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA22 STEM</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF1F8A82"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Lis Lowndes</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FFD98A3D"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA24 Visual Art</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FFD98A3D"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Natalie Carter</t>
     </r>
   </si>
   <si>
@@ -325,7 +1308,7 @@
         <color rgb="FF29A39A"/>
         <sz val="10"/>
       </rPr>
-      <t>LA17 STEM</t>
+      <t>LA6 STEM</t>
     </r>
     <r>
       <rPr>
@@ -333,6 +1316,28 @@
         <sz val="9"/>
       </rPr>
       <t xml:space="preserve">  Chantel Uhe</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FFD4538A"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA7 Performing Arts</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FFD4538A"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Cheryl Peak</t>
     </r>
     <r>
       <rPr>
@@ -347,7 +1352,7 @@
         <color rgb="FF1F8A82"/>
         <sz val="10"/>
       </rPr>
-      <t>LA14 STEM</t>
+      <t>LA18 STEM</t>
     </r>
     <r>
       <rPr>
@@ -356,15 +1361,142 @@
       </rPr>
       <t xml:space="preserve">  Lis Lowndes</t>
     </r>
-  </si>
-  <si>
+    <r>
+      <rPr>
+        <sz val="6"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FFD98A3D"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA16 Visual Art</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FFD98A3D"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Natalie Carter</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF29A39A"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA7 STEM</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF29A39A"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Chantel Uhe</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF7E57C2"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA9 Auslan</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF7E57C2"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Rachel Walker</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
     <r>
       <rPr>
         <b/>
         <color rgb="FF1F8A82"/>
         <sz val="10"/>
       </rPr>
-      <t>LA6 PE</t>
+      <t>LA19 STEM</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF1F8A82"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Lis Lowndes</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FFD98A3D"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA8 Visual Art</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FFD98A3D"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Natalie Carter</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FFD4538A"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA18 Performing Arts</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FFD4538A"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Cheryl Peak</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF1F8A82"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA18 PE</t>
     </r>
     <r>
       <rPr>
@@ -386,7 +1518,7 @@
         <color rgb="FF4A90D9"/>
         <sz val="10"/>
       </rPr>
-      <t>LA8 PE</t>
+      <t>LA19 PE</t>
     </r>
     <r>
       <rPr>
@@ -408,7 +1540,7 @@
         <color rgb="FF6AA9E0"/>
         <sz val="10"/>
       </rPr>
-      <t>LA9 PE</t>
+      <t>LA20 PE</t>
     </r>
     <r>
       <rPr>
@@ -430,7 +1562,7 @@
         <color rgb="FF7E57C2"/>
         <sz val="10"/>
       </rPr>
-      <t>LA14 Auslan</t>
+      <t>LA7 Auslan</t>
     </r>
     <r>
       <rPr>
@@ -452,7 +1584,7 @@
         <color rgb="FFD4538A"/>
         <sz val="10"/>
       </rPr>
-      <t>LA21 Performing Arts</t>
+      <t>LA24 Performing Arts</t>
     </r>
     <r>
       <rPr>
@@ -469,7 +1601,7 @@
         <color rgb="FFD4538A"/>
         <sz val="10"/>
       </rPr>
-      <t>LA18 Auslan</t>
+      <t>LA22 Auslan</t>
     </r>
     <r>
       <rPr>
@@ -491,7 +1623,7 @@
         <color rgb="FF1F8A82"/>
         <sz val="10"/>
       </rPr>
-      <t>LA15 STEM</t>
+      <t>LA21 STEM</t>
     </r>
     <r>
       <rPr>
@@ -513,7 +1645,7 @@
         <color rgb="FF4A90D9"/>
         <sz val="10"/>
       </rPr>
-      <t>LA21 Health</t>
+      <t>LA9 Health</t>
     </r>
     <r>
       <rPr>
@@ -524,8 +1656,15 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">P3
-10:25-11:10</t>
+    <t xml:space="preserve">Recess
+1:20-1:35</t>
+  </si>
+  <si>
+    <t>Recess (1:20-1:35)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P6
+1:35-2:35</t>
   </si>
   <si>
     <r>
@@ -534,7 +1673,7 @@
         <color rgb="FF1F8A82"/>
         <sz val="10"/>
       </rPr>
-      <t>LA20 STEM</t>
+      <t>LA22 STEM</t>
     </r>
     <r>
       <rPr>
@@ -542,6 +1681,28 @@
         <sz val="9"/>
       </rPr>
       <t xml:space="preserve">  Lis Lowndes</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FFD98A3D"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA17 Visual Art</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FFD98A3D"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Natalie Carter</t>
     </r>
   </si>
   <si>
@@ -551,7 +1712,7 @@
         <color rgb="FF29A39A"/>
         <sz val="10"/>
       </rPr>
-      <t>LA9 STEM</t>
+      <t>LA6 STEM</t>
     </r>
     <r>
       <rPr>
@@ -559,6 +1720,28 @@
         <sz val="9"/>
       </rPr>
       <t xml:space="preserve">  Chantel Uhe</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF1F8A82"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA18 STEM</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF1F8A82"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Lis Lowndes</t>
     </r>
     <r>
       <rPr>
@@ -573,7 +1756,7 @@
         <color rgb="FFD4538A"/>
         <sz val="10"/>
       </rPr>
-      <t>LA16 Performing Arts</t>
+      <t>LA14 Performing Arts</t>
     </r>
     <r>
       <rPr>
@@ -581,6 +1764,67 @@
         <sz val="9"/>
       </rPr>
       <t xml:space="preserve">  Cheryl Peak</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FFD98A3D"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA20 Visual Art</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FFD98A3D"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Natalie Carter</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF29A39A"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA7 STEM</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF29A39A"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Chantel Uhe</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF7E57C2"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA21 Auslan</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF7E57C2"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Rachel Walker</t>
     </r>
     <r>
       <rPr>
@@ -595,7 +1839,7 @@
         <color rgb="FF1F8A82"/>
         <sz val="10"/>
       </rPr>
-      <t>LA22 STEM</t>
+      <t>LA23 Health</t>
     </r>
     <r>
       <rPr>
@@ -603,6 +1847,28 @@
         <sz val="9"/>
       </rPr>
       <t xml:space="preserve">  Lis Lowndes</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FFD4538A"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA15 Performing Arts</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FFD4538A"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Cheryl Peak</t>
     </r>
     <r>
       <rPr>
@@ -617,7 +1883,7 @@
         <color rgb="FFD98A3D"/>
         <sz val="10"/>
       </rPr>
-      <t>LA14 Visual Art</t>
+      <t>LA9 Visual Art</t>
     </r>
     <r>
       <rPr>
@@ -631,17 +1897,83 @@
     <r>
       <rPr>
         <b/>
-        <color rgb="FF29A39A"/>
+        <color rgb="FF1F8A82"/>
         <sz val="10"/>
       </rPr>
-      <t>LA16 STEM</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FF29A39A"/>
+      <t>LA22 PE</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF1F8A82"/>
         <sz val="9"/>
       </rPr>
-      <t xml:space="preserve">  Chantel Uhe</t>
+      <t xml:space="preserve">  Lis Lowndes</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF4A90D9"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA23 PE</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF4A90D9"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Aaron Bell</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF6AA9E0"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA24 PE</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF6AA9E0"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Jake Pevitt</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF7E57C2"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA16 Auslan</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF7E57C2"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Rachel Walker</t>
     </r>
     <r>
       <rPr>
@@ -656,7 +1988,7 @@
         <color rgb="FFD4538A"/>
         <sz val="10"/>
       </rPr>
-      <t>LA6 Performing Arts</t>
+      <t>LA8 Performing Arts</t>
     </r>
     <r>
       <rPr>
@@ -665,88 +1997,22 @@
       </rPr>
       <t xml:space="preserve">  Cheryl Peak</t>
     </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
+  </si>
+  <si>
     <r>
       <rPr>
         <b/>
-        <color rgb="FF7E57C2"/>
+        <color rgb="FFD4538A"/>
         <sz val="10"/>
       </rPr>
-      <t>LA8 Auslan</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FF7E57C2"/>
+      <t>LA19 Auslan</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FFD4538A"/>
         <sz val="9"/>
       </rPr>
-      <t xml:space="preserve">  Rachel Walker</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF1F8A82"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA14 STEM</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FF1F8A82"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Lis Lowndes</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FFD98A3D"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA15 Visual Art</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FFD98A3D"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Natalie Carter</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF1F8A82"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA7 PE</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FF1F8A82"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Lis Lowndes</t>
+      <t xml:space="preserve">  Cheryl Peak</t>
     </r>
     <r>
       <rPr>
@@ -761,7 +2027,7 @@
         <color rgb="FF4A90D9"/>
         <sz val="10"/>
       </rPr>
-      <t>LA16 PE</t>
+      <t>LA24 Health</t>
     </r>
     <r>
       <rPr>
@@ -770,1294 +2036,6 @@
       </rPr>
       <t xml:space="preserve">  Aaron Bell</t>
     </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF6AA9E0"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA17 PE</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FF6AA9E0"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Jake Pevitt</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF7E57C2"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA15 Auslan</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FF7E57C2"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Rachel Walker</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FFD4538A"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA22 Performing Arts</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FFD4538A"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Cheryl Peak</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FFD4538A"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA20 Auslan</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FFD4538A"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Cheryl Peak</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF4A90D9"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA18 Health</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FF4A90D9"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Aaron Bell</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF1F8A82"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA15 STEM</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FF1F8A82"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Lis Lowndes</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">Lunch
-11:10-11:50</t>
-  </si>
-  <si>
-    <t>Lunch (11:10-11:50)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P4
-11:50-12:35</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF1F8A82"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA23 STEM</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FF1F8A82"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Lis Lowndes</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FFD98A3D"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA18 Visual Art</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FFD98A3D"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Natalie Carter</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF29A39A"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA9 STEM</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FF29A39A"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Chantel Uhe</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FFD4538A"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA17 Performing Arts</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FFD4538A"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Cheryl Peak</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF1F8A82"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA22 STEM</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FF1F8A82"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Lis Lowndes</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FFD98A3D"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA7 Visual Art</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FFD98A3D"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Natalie Carter</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF29A39A"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA16 STEM</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FF29A39A"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Chantel Uhe</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FFD98A3D"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA22 Visual Art</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FFD98A3D"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Natalie Carter</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FFD4538A"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA23 Performing Arts</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FFD4538A"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Cheryl Peak</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF7E57C2"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA24 Auslan</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FF7E57C2"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Rachel Walker</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF1F8A82"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA19 STEM</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FF1F8A82"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Lis Lowndes</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF1F8A82"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA14 PE</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FF1F8A82"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Lis Lowndes</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF4A90D9"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA15 PE</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FF4A90D9"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Aaron Bell</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF6AA9E0"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA21 PE</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FF6AA9E0"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Jake Pevitt</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF7E57C2"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA17 Auslan</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FF7E57C2"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Rachel Walker</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FFD4538A"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA19 Performing Arts</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FFD4538A"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Cheryl Peak</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FFD4538A"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA23 Auslan</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FFD4538A"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Cheryl Peak</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF4A90D9"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA22 Health</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FF4A90D9"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Aaron Bell</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF1F8A82"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA21 STEM</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FF1F8A82"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Lis Lowndes</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">P5
-12:35-1:20</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF1F8A82"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA23 STEM</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FF1F8A82"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Lis Lowndes</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FFD98A3D"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA24 Visual Art</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FFD98A3D"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Natalie Carter</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF29A39A"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA6 STEM</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FF29A39A"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Chantel Uhe</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FFD4538A"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA7 Performing Arts</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FFD4538A"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Cheryl Peak</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF1F8A82"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA18 STEM</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FF1F8A82"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Lis Lowndes</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FFD98A3D"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA16 Visual Art</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FFD98A3D"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Natalie Carter</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF29A39A"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA7 STEM</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FF29A39A"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Chantel Uhe</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF7E57C2"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA9 Auslan</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FF7E57C2"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Rachel Walker</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF1F8A82"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA19 STEM</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FF1F8A82"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Lis Lowndes</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FFD98A3D"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA8 Visual Art</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FFD98A3D"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Natalie Carter</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FFD4538A"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA18 Performing Arts</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FFD4538A"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Cheryl Peak</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF1F8A82"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA18 PE</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FF1F8A82"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Lis Lowndes</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF4A90D9"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA19 PE</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FF4A90D9"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Aaron Bell</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF6AA9E0"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA20 PE</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FF6AA9E0"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Jake Pevitt</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF7E57C2"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA7 Auslan</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FF7E57C2"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Rachel Walker</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FFD4538A"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA24 Performing Arts</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FFD4538A"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Cheryl Peak</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FFD4538A"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA22 Auslan</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FFD4538A"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Cheryl Peak</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF1F8A82"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA21 STEM</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FF1F8A82"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Lis Lowndes</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF4A90D9"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA9 Health</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FF4A90D9"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Aaron Bell</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">Recess
-1:20-1:35</t>
-  </si>
-  <si>
-    <t>Recess (1:20-1:35)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P6
-1:35-2:35</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FFD98A3D"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA17 Visual Art</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FFD98A3D"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Natalie Carter</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF29A39A"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA6 STEM</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FF29A39A"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Chantel Uhe</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF1F8A82"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA18 STEM</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FF1F8A82"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Lis Lowndes</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FFD4538A"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA14 Performing Arts</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FFD4538A"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Cheryl Peak</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FFD98A3D"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA20 Visual Art</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FFD98A3D"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Natalie Carter</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF29A39A"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA7 STEM</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FF29A39A"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Chantel Uhe</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF7E57C2"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA21 Auslan</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FF7E57C2"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Rachel Walker</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF1F8A82"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA23 Health</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FF1F8A82"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Lis Lowndes</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FFD4538A"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA15 Performing Arts</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FFD4538A"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Cheryl Peak</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FFD98A3D"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA9 Visual Art</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FFD98A3D"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Natalie Carter</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF1F8A82"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA22 PE</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FF1F8A82"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Lis Lowndes</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF4A90D9"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA23 PE</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FF4A90D9"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Aaron Bell</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF6AA9E0"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA24 PE</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FF6AA9E0"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Jake Pevitt</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF7E57C2"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA16 Auslan</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FF7E57C2"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Rachel Walker</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FFD4538A"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA8 Performing Arts</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FFD4538A"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Cheryl Peak</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FFD4538A"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA19 Auslan</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FFD4538A"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Cheryl Peak</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF4A90D9"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA24 Health</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FF4A90D9"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Aaron Bell</t>
-    </r>
   </si>
   <si>
     <t>Mon · whole school (specialist in colour, otherwise classroom teacher)</t>
@@ -2174,13 +2152,13 @@
     <t>P1 8:55-9:40</t>
   </si>
   <si>
-    <t>P2 9:40-10:25</t>
-  </si>
-  <si>
     <t xml:space="preserve">Visual Art
 Natalie Carter</t>
   </si>
   <si>
+    <t>P2 9:40-10:25</t>
+  </si>
+  <si>
     <t xml:space="preserve">STEM
 Lis Lowndes</t>
   </si>
@@ -2537,30 +2515,30 @@
 STEM</t>
   </si>
   <si>
+    <t xml:space="preserve">LA23 (1)
+STEM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LA7 (5)
+PE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LA19 (2)
+STEM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LA14 (3/4)
+PE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LA21 (3)
+STEM</t>
+  </si>
+  <si>
     <t xml:space="preserve">LA22 (1)
 STEM</t>
   </si>
   <si>
-    <t xml:space="preserve">LA7 (5)
-PE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LA23 (1)
-STEM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LA19 (2)
-STEM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LA14 (3/4)
-PE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LA21 (3)
-STEM</t>
-  </si>
-  <si>
     <t xml:space="preserve">LA18 (2)
 STEM</t>
   </si>
@@ -3028,7 +3006,7 @@
     <t>2. Period 6 reconciliation</t>
   </si>
   <si>
-    <t>Period 6 lessons: 17 · 15 base class releases + 2 graduate Health. Some Health periods are deliberately off Period 6: the two leadership-release Healths (LA9, LA21) and two grad Healths (LA18, LA22) sit in Friday P2-P5 (Aaron Bell; P1 is the assembly), since Bell only has one P6 slot. Every Years 1-6 class still has a Period 6 release.</t>
+    <t>Period 6 lessons: 18 · 16 base class releases + 2 graduate Health. Some Health periods are deliberately off Period 6: the two leadership-release Healths (LA9, LA21) and two grad Healths (LA18, LA22) sit in Friday P2-P5 (Aaron Bell; P1 is the assembly), since Bell only has one P6 slot. Every Years 1-6 class still has a Period 6 release.</t>
   </si>
   <si>
     <t>| Day | Class | Subject | Teacher | Type |</t>
@@ -3040,6 +3018,9 @@
     <t>| Mon | LA17 | Visual Art | Natalie Carter | base release |</t>
   </si>
   <si>
+    <t>| Mon | LA22 | STEM | Lis Lowndes | base release |</t>
+  </si>
+  <si>
     <t>| Tue | LA14 | Performing Arts | Cheryl Peak | base release |</t>
   </si>
   <si>
@@ -3115,7 +3096,7 @@
     <t>4. Monday P0 and P1 vacancy</t>
   </si>
   <si>
-    <t>Monday P0 specialist lessons: 0. Monday P1 specialist lessons: 0. Clear of all specialist activity: PASS.</t>
+    <t>Monday P0 specialist lessons: 0. Monday P1 specialist lessons: 1. Clear of all specialist activity: FAIL.</t>
   </si>
   <si>
     <t>5. DOTT equity</t>
@@ -3133,7 +3114,7 @@
     <t>| Chantel Uhe | 0.4 teach | 12 | 50m | 108m | by design (office days carry her DOTT) |</t>
   </si>
   <si>
-    <t>| Lis Lowndes | 1.0 | 24 | 425m | 270m | OK |</t>
+    <t>| Lis Lowndes | 1.0 | 24 | 410m | 270m | OK |</t>
   </si>
   <si>
     <t>| Natalie Carter | 0.6 | 15 | 165m | 162m | OK |</t>
@@ -3193,7 +3174,7 @@
     <t>| LA21 | Jasper Sirr-Davis | OHS | 285m +45 lead | 270m | +15 collab top-up; +45 leadership (separate) |</t>
   </si>
   <si>
-    <t>| LA22 | Imogen Webb | grad | 330m | 270m | +60m (grad extra Health) |</t>
+    <t>| LA22 | Imogen Webb | grad | 345m | 270m | +75m (grad extra Health) |</t>
   </si>
   <si>
     <t>| LA23 | Ashlee Hutchings | grad | 345m | 270m | +75m (grad extra Health) |</t>
@@ -3340,10 +3321,10 @@
     <t>| LA21 | 0 | 0 | 2 | 2 | 3 | 3 (incl leadership) |</t>
   </si>
   <si>
-    <t>| LA22 | 0 | 2 | 1 | 2 | 2 | 2 |</t>
-  </si>
-  <si>
-    <t>| LA23 | 2 | 1 | 2 | 1 | 1 | 2 |</t>
+    <t>| LA22 | 2 | 0 | 1 | 2 | 2 | 2 |</t>
+  </si>
+  <si>
+    <t>| LA23 | 1 | 2 | 2 | 1 | 1 | 2 |</t>
   </si>
   <si>
     <t>| LA24 | 1 | 2 | 1 | 2 | 1 | 2 |</t>
@@ -3382,7 +3363,7 @@
     <t>STEM (rule 5): every STEM block is two back-to-back periods (consecutive period numbers, same day): PASS.</t>
   </si>
   <si>
-    <t>Specialist teaching by period (rule 7 aims to keep mornings lighter for literacy): P1:7  P2:16  P3:18  P4:19  P5:19  P6:17. Note Thursday PE necessarily fills some morning slots; the rest of the week is pushed later where the other hard rules allow.</t>
+    <t>Specialist teaching by period (rule 7 aims to keep mornings lighter for literacy): P1:7  P2:16  P3:18  P4:18  P5:19  P6:18. Note Thursday PE necessarily fills some morning slots; the rest of the week is pushed later where the other hard rules allow.</t>
   </si>
   <si>
     <t>10. Pre-Primary &amp; Kindy DOTT ledger</t>
@@ -4048,7 +4029,7 @@
       <c r="E3" s="4"/>
       <c r="F3" s="4"/>
     </row>
-    <row r="4" ht="56" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" ht="40" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>9</v>
       </c>
@@ -4374,8 +4355,8 @@
       <c r="N4" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="O4" s="9" t="s">
-        <v>78</v>
+      <c r="O4" s="10" t="s">
+        <v>81</v>
       </c>
       <c r="P4" s="9" t="s">
         <v>79</v>
@@ -4383,10 +4364,10 @@
     </row>
     <row r="5" ht="32" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="B5" s="10" t="s">
         <v>81</v>
-      </c>
-      <c r="B5" s="10" t="s">
-        <v>82</v>
       </c>
       <c r="C5" s="9" t="s">
         <v>66</v>
@@ -4532,7 +4513,7 @@
         <v>72</v>
       </c>
       <c r="J8" s="10" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="K8" s="9" t="s">
         <v>74</v>
@@ -4546,8 +4527,8 @@
       <c r="N8" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="O8" s="11" t="s">
-        <v>83</v>
+      <c r="O8" s="9" t="s">
+        <v>78</v>
       </c>
       <c r="P8" s="9" t="s">
         <v>79</v>
@@ -4593,14 +4574,14 @@
       <c r="M9" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="N9" s="9" t="s">
-        <v>77</v>
-      </c>
-      <c r="O9" s="11" t="s">
+      <c r="N9" s="11" t="s">
         <v>83</v>
       </c>
+      <c r="O9" s="9" t="s">
+        <v>78</v>
+      </c>
       <c r="P9" s="10" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="10" ht="14" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
@@ -4651,7 +4632,7 @@
         <v>71</v>
       </c>
       <c r="I11" s="10" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J11" s="9" t="s">
         <v>73</v>
@@ -4665,8 +4646,8 @@
       <c r="M11" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="N11" s="9" t="s">
-        <v>77</v>
+      <c r="N11" s="11" t="s">
+        <v>83</v>
       </c>
       <c r="O11" s="9" t="s">
         <v>78</v>
@@ -4838,8 +4819,8 @@
       <c r="N16" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="O16" s="10" t="s">
-        <v>82</v>
+      <c r="O16" s="9" t="s">
+        <v>78</v>
       </c>
       <c r="P16" s="11" t="s">
         <v>83</v>
@@ -4847,7 +4828,7 @@
     </row>
     <row r="17" ht="32" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B17" s="9" t="s">
         <v>65</v>
@@ -4877,7 +4858,7 @@
         <v>73</v>
       </c>
       <c r="K17" s="10" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="L17" s="13" t="s">
         <v>92</v>
@@ -4912,7 +4893,7 @@
         <v>91</v>
       </c>
       <c r="F18" s="10" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G18" s="9" t="s">
         <v>70</v>
@@ -4935,11 +4916,11 @@
       <c r="M18" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="N18" s="11" t="s">
+      <c r="N18" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="O18" s="11" t="s">
         <v>83</v>
-      </c>
-      <c r="O18" s="9" t="s">
-        <v>78</v>
       </c>
       <c r="P18" s="9" t="s">
         <v>79</v>
@@ -4975,7 +4956,7 @@
         <v>65</v>
       </c>
       <c r="C20" s="10" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D20" s="9" t="s">
         <v>67</v>
@@ -5007,11 +4988,11 @@
       <c r="M20" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="N20" s="11" t="s">
+      <c r="N20" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="O20" s="11" t="s">
         <v>83</v>
-      </c>
-      <c r="O20" s="9" t="s">
-        <v>78</v>
       </c>
       <c r="P20" s="9" t="s">
         <v>79</v>
@@ -5040,7 +5021,7 @@
         <v>70</v>
       </c>
       <c r="H21" s="10" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="I21" s="9" t="s">
         <v>72</v>
@@ -5124,7 +5105,7 @@
         <v>74</v>
       </c>
       <c r="L23" s="10" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="M23" s="9" t="s">
         <v>76</v>
@@ -5297,7 +5278,7 @@
         <v>75</v>
       </c>
       <c r="M28" s="10" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="N28" s="9" t="s">
         <v>77</v>
@@ -5311,7 +5292,7 @@
     </row>
     <row r="29" ht="32" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A29" s="8" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B29" s="9" t="s">
         <v>65</v>
@@ -5379,7 +5360,7 @@
         <v>83</v>
       </c>
       <c r="G30" s="10" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="H30" s="12" t="s">
         <v>91</v>
@@ -5472,7 +5453,7 @@
         <v>76</v>
       </c>
       <c r="N32" s="10" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="O32" s="13" t="s">
         <v>92</v>
@@ -5492,7 +5473,7 @@
         <v>91</v>
       </c>
       <c r="D33" s="10" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="E33" s="14" t="s">
         <v>94</v>
@@ -5567,7 +5548,7 @@
         <v>67</v>
       </c>
       <c r="E35" s="10" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F35" s="9" t="s">
         <v>69</v>
@@ -5775,7 +5756,7 @@
     </row>
     <row r="41" ht="32" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A41" s="8" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B41" s="11" t="s">
         <v>97</v>
@@ -6239,7 +6220,7 @@
     </row>
     <row r="53" ht="32" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A53" s="8" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B53" s="9" t="s">
         <v>65</v>
@@ -6635,10 +6616,10 @@
     </row>
     <row r="5" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="B5" s="10" t="s">
         <v>81</v>
-      </c>
-      <c r="B5" s="10" t="s">
-        <v>82</v>
       </c>
       <c r="C5" s="9" t="s">
         <v>65</v>
@@ -6829,7 +6810,7 @@
     </row>
     <row r="17" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B17" s="9" t="s">
         <v>66</v>
@@ -6887,7 +6868,7 @@
         <v>66</v>
       </c>
       <c r="C20" s="10" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D20" s="9" t="s">
         <v>66</v>
@@ -7023,7 +7004,7 @@
     </row>
     <row r="29" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="8" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B29" s="9" t="s">
         <v>67</v>
@@ -7104,7 +7085,7 @@
         <v>67</v>
       </c>
       <c r="D33" s="10" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="E33" s="9" t="s">
         <v>67</v>
@@ -7217,7 +7198,7 @@
     </row>
     <row r="41" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" s="8" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B41" s="9" t="s">
         <v>68</v>
@@ -7330,7 +7311,7 @@
         <v>68</v>
       </c>
       <c r="D47" s="10" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="E47" s="9" t="s">
         <v>68</v>
@@ -7411,7 +7392,7 @@
     </row>
     <row r="53" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" s="8" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B53" s="9" t="s">
         <v>69</v>
@@ -7437,7 +7418,7 @@
         <v>69</v>
       </c>
       <c r="C54" s="10" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D54" s="11" t="s">
         <v>83</v>
@@ -7605,7 +7586,7 @@
     </row>
     <row r="65" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="8" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B65" s="9" t="s">
         <v>70</v>
@@ -7634,7 +7615,7 @@
         <v>70</v>
       </c>
       <c r="D66" s="10" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="E66" s="14" t="s">
         <v>94</v>
@@ -7799,7 +7780,7 @@
     </row>
     <row r="77" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A77" s="8" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B77" s="9" t="s">
         <v>71</v>
@@ -7877,7 +7858,7 @@
         <v>71</v>
       </c>
       <c r="C81" s="10" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D81" s="9" t="s">
         <v>71</v>
@@ -7993,7 +7974,7 @@
     </row>
     <row r="89" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A89" s="8" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B89" s="9" t="s">
         <v>72</v>
@@ -8100,7 +8081,7 @@
         <v>89</v>
       </c>
       <c r="B95" s="10" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C95" s="9" t="s">
         <v>72</v>
@@ -8187,7 +8168,7 @@
     </row>
     <row r="101" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A101" s="8" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B101" s="9" t="s">
         <v>73</v>
@@ -8242,7 +8223,7 @@
         <v>86</v>
       </c>
       <c r="B104" s="10" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C104" s="9" t="s">
         <v>73</v>
@@ -8381,13 +8362,13 @@
     </row>
     <row r="113" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A113" s="8" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B113" s="9" t="s">
         <v>74</v>
       </c>
       <c r="C113" s="10" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D113" s="9" t="s">
         <v>74</v>
@@ -8575,7 +8556,7 @@
     </row>
     <row r="125" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A125" s="8" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B125" s="11" t="s">
         <v>83</v>
@@ -8685,7 +8666,7 @@
         <v>75</v>
       </c>
       <c r="C131" s="10" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D131" s="9" t="s">
         <v>75</v>
@@ -8758,7 +8739,7 @@
         <v>76</v>
       </c>
       <c r="D136" s="10" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="E136" s="9" t="s">
         <v>76</v>
@@ -8769,7 +8750,7 @@
     </row>
     <row r="137" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A137" s="8" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B137" s="9" t="s">
         <v>76</v>
@@ -8963,7 +8944,7 @@
     </row>
     <row r="149" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A149" s="8" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B149" s="9" t="s">
         <v>77</v>
@@ -8988,8 +8969,8 @@
       <c r="B150" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="C150" s="11" t="s">
-        <v>83</v>
+      <c r="C150" s="9" t="s">
+        <v>77</v>
       </c>
       <c r="D150" s="9" t="s">
         <v>77</v>
@@ -9020,11 +9001,11 @@
       <c r="B152" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="C152" s="11" t="s">
-        <v>83</v>
+      <c r="C152" s="9" t="s">
+        <v>77</v>
       </c>
       <c r="D152" s="10" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="E152" s="9" t="s">
         <v>77</v>
@@ -9037,8 +9018,8 @@
       <c r="A153" s="8" t="s">
         <v>87</v>
       </c>
-      <c r="B153" s="9" t="s">
-        <v>77</v>
+      <c r="B153" s="11" t="s">
+        <v>83</v>
       </c>
       <c r="C153" s="9" t="s">
         <v>77</v>
@@ -9069,8 +9050,8 @@
       <c r="A155" s="8" t="s">
         <v>89</v>
       </c>
-      <c r="B155" s="9" t="s">
-        <v>77</v>
+      <c r="B155" s="11" t="s">
+        <v>83</v>
       </c>
       <c r="C155" s="9" t="s">
         <v>77</v>
@@ -9139,11 +9120,11 @@
       <c r="A160" s="8" t="s">
         <v>80</v>
       </c>
-      <c r="B160" s="9" t="s">
+      <c r="B160" s="10" t="s">
+        <v>81</v>
+      </c>
+      <c r="C160" s="9" t="s">
         <v>78</v>
-      </c>
-      <c r="C160" s="10" t="s">
-        <v>82</v>
       </c>
       <c r="D160" s="9" t="s">
         <v>78</v>
@@ -9157,7 +9138,7 @@
     </row>
     <row r="161" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A161" s="8" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B161" s="9" t="s">
         <v>78</v>
@@ -9182,8 +9163,8 @@
       <c r="B162" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="C162" s="9" t="s">
-        <v>78</v>
+      <c r="C162" s="11" t="s">
+        <v>83</v>
       </c>
       <c r="D162" s="9" t="s">
         <v>78</v>
@@ -9211,11 +9192,11 @@
       <c r="A164" s="8" t="s">
         <v>86</v>
       </c>
-      <c r="B164" s="11" t="s">
+      <c r="B164" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="C164" s="11" t="s">
         <v>83</v>
-      </c>
-      <c r="C164" s="9" t="s">
-        <v>78</v>
       </c>
       <c r="D164" s="13" t="s">
         <v>92</v>
@@ -9231,8 +9212,8 @@
       <c r="A165" s="8" t="s">
         <v>87</v>
       </c>
-      <c r="B165" s="11" t="s">
-        <v>83</v>
+      <c r="B165" s="9" t="s">
+        <v>78</v>
       </c>
       <c r="C165" s="9" t="s">
         <v>78</v>
@@ -9351,7 +9332,7 @@
     </row>
     <row r="173" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A173" s="8" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B173" s="9" t="s">
         <v>79</v>
@@ -9426,7 +9407,7 @@
         <v>87</v>
       </c>
       <c r="B177" s="10" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C177" s="9" t="s">
         <v>79</v>
@@ -9607,7 +9588,7 @@
     </row>
     <row r="5" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B5" s="17" t="s">
         <v>121</v>
@@ -9801,7 +9782,7 @@
     </row>
     <row r="17" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B17" s="9" t="s">
         <v>126</v>
@@ -9995,7 +9976,7 @@
     </row>
     <row r="29" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="8" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B29" s="9" t="s">
         <v>129</v>
@@ -10189,7 +10170,7 @@
     </row>
     <row r="41" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" s="8" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B41" s="9" t="s">
         <v>131</v>
@@ -10383,7 +10364,7 @@
     </row>
     <row r="53" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" s="8" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B53" s="9" t="s">
         <v>134</v>
@@ -10577,7 +10558,7 @@
     </row>
     <row r="65" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="8" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B65" s="9" t="s">
         <v>138</v>
@@ -10771,7 +10752,7 @@
     </row>
     <row r="77" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A77" s="8" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B77" s="9" t="s">
         <v>140</v>
@@ -10965,7 +10946,7 @@
     </row>
     <row r="89" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A89" s="8" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B89" s="9" t="s">
         <v>142</v>
@@ -11159,7 +11140,7 @@
     </row>
     <row r="101" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A101" s="8" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B101" s="9" t="s">
         <v>144</v>
@@ -11353,7 +11334,7 @@
     </row>
     <row r="113" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A113" s="8" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B113" s="9" t="s">
         <v>149</v>
@@ -11547,7 +11528,7 @@
     </row>
     <row r="125" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A125" s="8" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B125" s="17" t="s">
         <v>135</v>
@@ -11741,7 +11722,7 @@
     </row>
     <row r="137" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A137" s="8" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B137" s="9" t="s">
         <v>153</v>
@@ -11935,7 +11916,7 @@
     </row>
     <row r="149" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A149" s="8" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B149" s="9" t="s">
         <v>156</v>
@@ -11960,8 +11941,8 @@
       <c r="B150" s="9" t="s">
         <v>156</v>
       </c>
-      <c r="C150" s="17" t="s">
-        <v>135</v>
+      <c r="C150" s="9" t="s">
+        <v>156</v>
       </c>
       <c r="D150" s="9" t="s">
         <v>156</v>
@@ -11992,8 +11973,8 @@
       <c r="B152" s="9" t="s">
         <v>156</v>
       </c>
-      <c r="C152" s="17" t="s">
-        <v>135</v>
+      <c r="C152" s="9" t="s">
+        <v>156</v>
       </c>
       <c r="D152" s="18" t="s">
         <v>157</v>
@@ -12009,8 +11990,8 @@
       <c r="A153" s="8" t="s">
         <v>87</v>
       </c>
-      <c r="B153" s="9" t="s">
-        <v>156</v>
+      <c r="B153" s="17" t="s">
+        <v>135</v>
       </c>
       <c r="C153" s="9" t="s">
         <v>156</v>
@@ -12041,8 +12022,8 @@
       <c r="A155" s="8" t="s">
         <v>89</v>
       </c>
-      <c r="B155" s="9" t="s">
-        <v>156</v>
+      <c r="B155" s="17" t="s">
+        <v>135</v>
       </c>
       <c r="C155" s="9" t="s">
         <v>156</v>
@@ -12111,11 +12092,11 @@
       <c r="A160" s="8" t="s">
         <v>80</v>
       </c>
-      <c r="B160" s="9" t="s">
+      <c r="B160" s="17" t="s">
+        <v>121</v>
+      </c>
+      <c r="C160" s="9" t="s">
         <v>160</v>
-      </c>
-      <c r="C160" s="17" t="s">
-        <v>121</v>
       </c>
       <c r="D160" s="9" t="s">
         <v>160</v>
@@ -12129,7 +12110,7 @@
     </row>
     <row r="161" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A161" s="8" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B161" s="9" t="s">
         <v>160</v>
@@ -12154,8 +12135,8 @@
       <c r="B162" s="9" t="s">
         <v>160</v>
       </c>
-      <c r="C162" s="9" t="s">
-        <v>160</v>
+      <c r="C162" s="17" t="s">
+        <v>135</v>
       </c>
       <c r="D162" s="9" t="s">
         <v>160</v>
@@ -12183,11 +12164,11 @@
       <c r="A164" s="8" t="s">
         <v>86</v>
       </c>
-      <c r="B164" s="17" t="s">
+      <c r="B164" s="9" t="s">
+        <v>160</v>
+      </c>
+      <c r="C164" s="17" t="s">
         <v>135</v>
-      </c>
-      <c r="C164" s="9" t="s">
-        <v>160</v>
       </c>
       <c r="D164" s="18" t="s">
         <v>157</v>
@@ -12203,8 +12184,8 @@
       <c r="A165" s="8" t="s">
         <v>87</v>
       </c>
-      <c r="B165" s="17" t="s">
-        <v>135</v>
+      <c r="B165" s="9" t="s">
+        <v>160</v>
       </c>
       <c r="C165" s="9" t="s">
         <v>160</v>
@@ -12323,7 +12304,7 @@
     </row>
     <row r="173" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A173" s="8" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B173" s="9" t="s">
         <v>164</v>
@@ -12517,7 +12498,7 @@
     </row>
     <row r="185" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A185" s="8" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B185" s="20" t="s">
         <v>167</v>
@@ -12711,7 +12692,7 @@
     </row>
     <row r="197" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A197" s="8" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B197" s="11" t="s">
         <v>179</v>
@@ -12765,20 +12746,20 @@
       <c r="A200" s="8" t="s">
         <v>86</v>
       </c>
-      <c r="B200" s="11" t="s">
-        <v>185</v>
+      <c r="B200" s="21" t="s">
+        <v>168</v>
       </c>
       <c r="C200" s="11" t="s">
         <v>183</v>
       </c>
       <c r="D200" s="11" t="s">
+        <v>185</v>
+      </c>
+      <c r="E200" s="11" t="s">
         <v>186</v>
       </c>
-      <c r="E200" s="11" t="s">
+      <c r="F200" s="11" t="s">
         <v>187</v>
-      </c>
-      <c r="F200" s="11" t="s">
-        <v>188</v>
       </c>
     </row>
     <row r="201" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -12786,19 +12767,19 @@
         <v>87</v>
       </c>
       <c r="B201" s="11" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="C201" s="11" t="s">
         <v>189</v>
       </c>
       <c r="D201" s="11" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="E201" s="11" t="s">
         <v>190</v>
       </c>
       <c r="F201" s="11" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="202" ht="14" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -12817,8 +12798,8 @@
       <c r="A203" s="8" t="s">
         <v>89</v>
       </c>
-      <c r="B203" s="21" t="s">
-        <v>168</v>
+      <c r="B203" s="11" t="s">
+        <v>188</v>
       </c>
       <c r="C203" s="11" t="s">
         <v>189</v>
@@ -12887,11 +12868,11 @@
       <c r="A208" s="8" t="s">
         <v>80</v>
       </c>
-      <c r="B208" s="21" t="s">
+      <c r="B208" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="C208" s="21" t="s">
         <v>168</v>
-      </c>
-      <c r="C208" s="10" t="s">
-        <v>195</v>
       </c>
       <c r="D208" s="10" t="s">
         <v>196</v>
@@ -12905,7 +12886,7 @@
     </row>
     <row r="209" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A209" s="8" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B209" s="10" t="s">
         <v>197</v>
@@ -13099,7 +13080,7 @@
     </row>
     <row r="221" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A221" s="8" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B221" s="20" t="s">
         <v>169</v>
@@ -13293,7 +13274,7 @@
     </row>
     <row r="233" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A233" s="8" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B233" s="20" t="s">
         <v>169</v>
@@ -13487,7 +13468,7 @@
     </row>
     <row r="245" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A245" s="8" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B245" s="20" t="s">
         <v>169</v>
@@ -13681,7 +13662,7 @@
     </row>
     <row r="257" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A257" s="8" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B257" s="20" t="s">
         <v>169</v>
@@ -13968,7 +13949,7 @@
     </row>
     <row r="7" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B7" s="9" t="s">
         <v>264</v>
@@ -14162,7 +14143,7 @@
     </row>
     <row r="19" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B19" s="9" t="s">
         <v>266</v>
@@ -14356,7 +14337,7 @@
     </row>
     <row r="31" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" s="8" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B31" s="9" t="s">
         <v>268</v>
@@ -14550,7 +14531,7 @@
     </row>
     <row r="43" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" s="8" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B43" s="20" t="s">
         <v>169</v>
@@ -14744,7 +14725,7 @@
     </row>
     <row r="55" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" s="8" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B55" s="9" t="s">
         <v>271</v>
@@ -14938,7 +14919,7 @@
     </row>
     <row r="67" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="8" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B67" s="9" t="s">
         <v>274</v>
@@ -15132,7 +15113,7 @@
     </row>
     <row r="79" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A79" s="8" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B79" s="20" t="s">
         <v>169</v>
@@ -15326,7 +15307,7 @@
     </row>
     <row r="91" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A91" s="8" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B91" s="21" t="s">
         <v>168</v>
@@ -15520,7 +15501,7 @@
     </row>
     <row r="103" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A103" s="8" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B103" s="9" t="s">
         <v>283</v>
@@ -15714,7 +15695,7 @@
     </row>
     <row r="115" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A115" s="8" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B115" s="9" t="s">
         <v>287</v>
@@ -15908,7 +15889,7 @@
     </row>
     <row r="127" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A127" s="8" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B127" s="9" t="s">
         <v>290</v>
@@ -16102,7 +16083,7 @@
     </row>
     <row r="139" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A139" s="8" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B139" s="20" t="s">
         <v>293</v>
@@ -16296,7 +16277,7 @@
     </row>
     <row r="151" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A151" s="8" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B151" s="9" t="s">
         <v>291</v>
@@ -16490,7 +16471,7 @@
     </row>
     <row r="163" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A163" s="8" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B163" s="20" t="s">
         <v>293</v>
@@ -16684,7 +16665,7 @@
     </row>
     <row r="175" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A175" s="8" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B175" s="9" t="s">
         <v>288</v>
@@ -16951,7 +16932,7 @@
     </row>
     <row r="7" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B7" s="9" t="s">
         <v>264</v>
@@ -17145,7 +17126,7 @@
     </row>
     <row r="19" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B19" s="9" t="s">
         <v>266</v>
@@ -17339,7 +17320,7 @@
     </row>
     <row r="31" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" s="8" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B31" s="9" t="s">
         <v>268</v>
@@ -17533,7 +17514,7 @@
     </row>
     <row r="43" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" s="8" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B43" s="20" t="s">
         <v>169</v>
@@ -17727,7 +17708,7 @@
     </row>
     <row r="55" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" s="8" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B55" s="9" t="s">
         <v>271</v>
@@ -17921,7 +17902,7 @@
     </row>
     <row r="67" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="8" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B67" s="9" t="s">
         <v>274</v>
@@ -18115,7 +18096,7 @@
     </row>
     <row r="79" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A79" s="8" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B79" s="20" t="s">
         <v>169</v>
@@ -18309,7 +18290,7 @@
     </row>
     <row r="91" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A91" s="8" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B91" s="21" t="s">
         <v>168</v>
@@ -18503,7 +18484,7 @@
     </row>
     <row r="103" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A103" s="8" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B103" s="9" t="s">
         <v>283</v>
@@ -18697,7 +18678,7 @@
     </row>
     <row r="115" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A115" s="8" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B115" s="9" t="s">
         <v>287</v>
@@ -18891,7 +18872,7 @@
     </row>
     <row r="127" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A127" s="8" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B127" s="9" t="s">
         <v>290</v>
@@ -19085,7 +19066,7 @@
     </row>
     <row r="139" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A139" s="8" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B139" s="20" t="s">
         <v>293</v>
@@ -19279,7 +19260,7 @@
     </row>
     <row r="151" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A151" s="8" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B151" s="9" t="s">
         <v>291</v>
@@ -19473,7 +19454,7 @@
     </row>
     <row r="163" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A163" s="8" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B163" s="20" t="s">
         <v>293</v>
@@ -19667,7 +19648,7 @@
     </row>
     <row r="175" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A175" s="8" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B175" s="9" t="s">
         <v>288</v>
@@ -19845,7 +19826,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A168"/>
+  <dimension ref="A1:A169"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="110" customWidth="1"/>
@@ -20037,38 +20018,38 @@
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
+      <c r="A38" s="24" t="s">
         <v>335</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
         <v>302</v>
       </c>
     </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A40" s="23" t="s">
-        <v>336</v>
-      </c>
-    </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A41" t="s">
+      <c r="A41" s="23" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
         <v>302</v>
-      </c>
-    </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A42" s="24" t="s">
-        <v>337</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A43" s="24" t="s">
-        <v>306</v>
+        <v>338</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A44" s="24" t="s">
-        <v>338</v>
+        <v>306</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.25">
@@ -20087,52 +20068,52 @@
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A48" t="s">
+      <c r="A48" s="24" t="s">
         <v>342</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
         <v>302</v>
       </c>
     </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A50" s="23" t="s">
-        <v>343</v>
-      </c>
-    </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A51" t="s">
-        <v>302</v>
+      <c r="A51" s="23" t="s">
+        <v>344</v>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>344</v>
+        <v>302</v>
       </c>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="54" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
         <v>302</v>
       </c>
     </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A54" s="23" t="s">
-        <v>345</v>
-      </c>
-    </row>
     <row r="55" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A55" t="s">
-        <v>302</v>
+      <c r="A55" s="23" t="s">
+        <v>346</v>
       </c>
     </row>
     <row r="56" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>346</v>
+        <v>302</v>
       </c>
     </row>
     <row r="57" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A57" s="24" t="s">
+      <c r="A57" t="s">
         <v>347</v>
       </c>
     </row>
@@ -20177,23 +20158,23 @@
       </c>
     </row>
     <row r="66" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A66" t="s">
+      <c r="A66" s="24" t="s">
         <v>356</v>
       </c>
     </row>
     <row r="67" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A67" s="24" t="s">
+      <c r="A67" t="s">
         <v>357</v>
       </c>
     </row>
     <row r="68" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A68" s="24" t="s">
-        <v>348</v>
+        <v>358</v>
       </c>
     </row>
     <row r="69" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A69" s="24" t="s">
-        <v>358</v>
+        <v>349</v>
       </c>
     </row>
     <row r="70" spans="1:1" x14ac:dyDescent="0.25">
@@ -20267,38 +20248,38 @@
       </c>
     </row>
     <row r="84" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A84" t="s">
+      <c r="A84" s="24" t="s">
         <v>373</v>
       </c>
     </row>
     <row r="85" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="86" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
         <v>302</v>
       </c>
     </row>
-    <row r="86" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A86" s="23" t="s">
-        <v>374</v>
-      </c>
-    </row>
     <row r="87" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A87" t="s">
+      <c r="A87" s="23" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="88" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
         <v>302</v>
-      </c>
-    </row>
-    <row r="88" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A88" s="24" t="s">
-        <v>375</v>
       </c>
     </row>
     <row r="89" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A89" s="24" t="s">
-        <v>306</v>
+        <v>376</v>
       </c>
     </row>
     <row r="90" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A90" s="24" t="s">
-        <v>376</v>
+        <v>306</v>
       </c>
     </row>
     <row r="91" spans="1:1" x14ac:dyDescent="0.25">
@@ -20332,28 +20313,28 @@
       </c>
     </row>
     <row r="97" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A97" t="s">
+      <c r="A97" s="24" t="s">
         <v>383</v>
       </c>
     </row>
     <row r="98" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="99" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
         <v>302</v>
       </c>
     </row>
-    <row r="99" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A99" s="23" t="s">
-        <v>384</v>
-      </c>
-    </row>
     <row r="100" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A100" t="s">
+      <c r="A100" s="23" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="101" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
         <v>302</v>
-      </c>
-    </row>
-    <row r="101" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A101" s="24" t="s">
-        <v>385</v>
       </c>
     </row>
     <row r="102" spans="1:1" x14ac:dyDescent="0.25">
@@ -20437,32 +20418,32 @@
       </c>
     </row>
     <row r="118" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A118" t="s">
+      <c r="A118" s="24" t="s">
         <v>402</v>
       </c>
     </row>
     <row r="119" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="120" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A120" t="s">
         <v>302</v>
       </c>
     </row>
-    <row r="120" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A120" s="23" t="s">
-        <v>403</v>
-      </c>
-    </row>
     <row r="121" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A121" t="s">
-        <v>302</v>
+      <c r="A121" s="23" t="s">
+        <v>404</v>
       </c>
     </row>
     <row r="122" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
-        <v>404</v>
+        <v>302</v>
       </c>
     </row>
     <row r="123" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A123" s="24" t="s">
+      <c r="A123" t="s">
         <v>405</v>
       </c>
     </row>
@@ -20547,32 +20528,32 @@
       </c>
     </row>
     <row r="140" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A140" t="s">
+      <c r="A140" s="24" t="s">
         <v>422</v>
       </c>
     </row>
     <row r="141" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="142" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A142" t="s">
         <v>302</v>
       </c>
     </row>
-    <row r="142" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A142" s="23" t="s">
-        <v>423</v>
-      </c>
-    </row>
     <row r="143" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A143" t="s">
-        <v>302</v>
+      <c r="A143" s="23" t="s">
+        <v>424</v>
       </c>
     </row>
     <row r="144" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
-        <v>424</v>
+        <v>302</v>
       </c>
     </row>
     <row r="145" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A145" s="24" t="s">
+      <c r="A145" t="s">
         <v>425</v>
       </c>
     </row>
@@ -20607,7 +20588,7 @@
       </c>
     </row>
     <row r="152" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A152" t="s">
+      <c r="A152" s="24" t="s">
         <v>432</v>
       </c>
     </row>
@@ -20618,37 +20599,37 @@
     </row>
     <row r="154" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="155" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A155" t="s">
         <v>302</v>
       </c>
     </row>
-    <row r="155" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A155" s="23" t="s">
-        <v>434</v>
-      </c>
-    </row>
     <row r="156" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A156" t="s">
-        <v>302</v>
+      <c r="A156" s="23" t="s">
+        <v>435</v>
       </c>
     </row>
     <row r="157" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
-        <v>435</v>
+        <v>302</v>
       </c>
     </row>
     <row r="158" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A158" s="24" t="s">
+      <c r="A158" t="s">
         <v>436</v>
       </c>
     </row>
     <row r="159" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A159" s="24" t="s">
-        <v>406</v>
+        <v>437</v>
       </c>
     </row>
     <row r="160" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A160" s="24" t="s">
-        <v>437</v>
+        <v>407</v>
       </c>
     </row>
     <row r="161" spans="1:1" x14ac:dyDescent="0.25">
@@ -20687,8 +20668,13 @@
       </c>
     </row>
     <row r="168" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A168" t="s">
+      <c r="A168" s="24" t="s">
         <v>445</v>
+      </c>
+    </row>
+    <row r="169" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A169" t="s">
+        <v>446</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
DOTT equity: close Nikki Luca's shortfall via Lis Friday cover
Move LA15 STEM (and LA20) to Monday to free Lis's Friday; Lis covers
Nikki's LA1 at Fri P2-P3 (2x45) instead of P6. Nikki -23 -> +7;
Lis +80 -> +50. No clashes; Friday P1 assembly still clear.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Tapping_S2_Specialist_Timetable.xlsx
+++ b/Tapping_S2_Specialist_Timetable.xlsx
@@ -466,10 +466,236 @@
     <r>
       <rPr>
         <b/>
+        <color rgb="FF4A90D9"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA21 Health</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF4A90D9"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Aaron Bell</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">P3
+10:25-11:10</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
         <color rgb="FF1F8A82"/>
         <sz val="10"/>
       </rPr>
       <t>LA15 STEM</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF1F8A82"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Lis Lowndes</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF29A39A"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA9 STEM</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF29A39A"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Chantel Uhe</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FFD4538A"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA16 Performing Arts</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FFD4538A"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Cheryl Peak</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF1F8A82"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA23 STEM</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF1F8A82"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Lis Lowndes</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FFD98A3D"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA14 Visual Art</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FFD98A3D"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Natalie Carter</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF29A39A"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA16 STEM</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF29A39A"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Chantel Uhe</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FFD4538A"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA6 Performing Arts</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FFD4538A"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Cheryl Peak</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF7E57C2"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA8 Auslan</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF7E57C2"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Rachel Walker</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF1F8A82"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA14 STEM</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF1F8A82"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Lis Lowndes</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FFD98A3D"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA15 Visual Art</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FFD98A3D"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Natalie Carter</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF1F8A82"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA7 PE</t>
     </r>
     <r>
       <rPr>
@@ -491,7 +717,7 @@
         <color rgb="FF4A90D9"/>
         <sz val="10"/>
       </rPr>
-      <t>LA21 Health</t>
+      <t>LA16 PE</t>
     </r>
     <r>
       <rPr>
@@ -500,10 +726,122 @@
       </rPr>
       <t xml:space="preserve">  Aaron Bell</t>
     </r>
-  </si>
-  <si>
-    <t xml:space="preserve">P3
-10:25-11:10</t>
+    <r>
+      <rPr>
+        <sz val="6"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF6AA9E0"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA17 PE</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF6AA9E0"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Jake Pevitt</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF7E57C2"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA15 Auslan</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF7E57C2"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Rachel Walker</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FFD4538A"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA22 Performing Arts</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FFD4538A"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Cheryl Peak</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FFD4538A"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA20 Auslan</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FFD4538A"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Cheryl Peak</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF4A90D9"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA18 Health</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF4A90D9"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Aaron Bell</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Lunch
+11:10-11:50</t>
+  </si>
+  <si>
+    <t>Lunch (11:10-11:50)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P4
+11:50-12:35</t>
   </si>
   <si>
     <r>
@@ -512,7 +850,7 @@
         <color rgb="FF1F8A82"/>
         <sz val="10"/>
       </rPr>
-      <t>LA20 STEM</t>
+      <t>LA15 STEM</t>
     </r>
     <r>
       <rPr>
@@ -520,6 +858,28 @@
         <sz val="9"/>
       </rPr>
       <t xml:space="preserve">  Lis Lowndes</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FFD98A3D"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA18 Visual Art</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FFD98A3D"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Natalie Carter</t>
     </r>
   </si>
   <si>
@@ -551,7 +911,7 @@
         <color rgb="FFD4538A"/>
         <sz val="10"/>
       </rPr>
-      <t>LA16 Performing Arts</t>
+      <t>LA17 Performing Arts</t>
     </r>
     <r>
       <rPr>
@@ -595,7 +955,7 @@
         <color rgb="FFD98A3D"/>
         <sz val="10"/>
       </rPr>
-      <t>LA14 Visual Art</t>
+      <t>LA7 Visual Art</t>
     </r>
     <r>
       <rPr>
@@ -631,10 +991,32 @@
     <r>
       <rPr>
         <b/>
+        <color rgb="FFD98A3D"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA22 Visual Art</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FFD98A3D"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Natalie Carter</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
         <color rgb="FFD4538A"/>
         <sz val="10"/>
       </rPr>
-      <t>LA6 Performing Arts</t>
+      <t>LA23 Performing Arts</t>
     </r>
     <r>
       <rPr>
@@ -656,7 +1038,7 @@
         <color rgb="FF7E57C2"/>
         <sz val="10"/>
       </rPr>
-      <t>LA8 Auslan</t>
+      <t>LA24 Auslan</t>
     </r>
     <r>
       <rPr>
@@ -678,7 +1060,194 @@
         <color rgb="FF1F8A82"/>
         <sz val="10"/>
       </rPr>
-      <t>LA14 STEM</t>
+      <t>LA19 STEM</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF1F8A82"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Lis Lowndes</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF1F8A82"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA14 PE</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF1F8A82"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Lis Lowndes</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF4A90D9"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA15 PE</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF4A90D9"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Aaron Bell</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF6AA9E0"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA21 PE</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF6AA9E0"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Jake Pevitt</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF7E57C2"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA17 Auslan</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF7E57C2"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Rachel Walker</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FFD4538A"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA19 Performing Arts</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FFD4538A"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Cheryl Peak</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FFD4538A"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA23 Auslan</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FFD4538A"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Cheryl Peak</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF4A90D9"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA22 Health</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF4A90D9"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Aaron Bell</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF1F8A82"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA21 STEM</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF1F8A82"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Lis Lowndes</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">P5
+12:35-1:20</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF1F8A82"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA22 STEM</t>
     </r>
     <r>
       <rPr>
@@ -700,7 +1269,7 @@
         <color rgb="FFD98A3D"/>
         <sz val="10"/>
       </rPr>
-      <t>LA15 Visual Art</t>
+      <t>LA24 Visual Art</t>
     </r>
     <r>
       <rPr>
@@ -711,13 +1280,201 @@
     </r>
   </si>
   <si>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF29A39A"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA6 STEM</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF29A39A"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Chantel Uhe</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FFD4538A"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA7 Performing Arts</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FFD4538A"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Cheryl Peak</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
     <r>
       <rPr>
         <b/>
         <color rgb="FF1F8A82"/>
         <sz val="10"/>
       </rPr>
-      <t>LA7 PE</t>
+      <t>LA18 STEM</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF1F8A82"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Lis Lowndes</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FFD98A3D"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA16 Visual Art</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FFD98A3D"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Natalie Carter</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF29A39A"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA7 STEM</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF29A39A"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Chantel Uhe</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF7E57C2"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA9 Auslan</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF7E57C2"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Rachel Walker</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF1F8A82"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA19 STEM</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF1F8A82"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Lis Lowndes</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FFD98A3D"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA8 Visual Art</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FFD98A3D"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Natalie Carter</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FFD4538A"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA18 Performing Arts</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FFD4538A"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Cheryl Peak</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF1F8A82"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA18 PE</t>
     </r>
     <r>
       <rPr>
@@ -739,7 +1496,7 @@
         <color rgb="FF4A90D9"/>
         <sz val="10"/>
       </rPr>
-      <t>LA16 PE</t>
+      <t>LA19 PE</t>
     </r>
     <r>
       <rPr>
@@ -761,7 +1518,7 @@
         <color rgb="FF6AA9E0"/>
         <sz val="10"/>
       </rPr>
-      <t>LA17 PE</t>
+      <t>LA20 PE</t>
     </r>
     <r>
       <rPr>
@@ -783,7 +1540,7 @@
         <color rgb="FF7E57C2"/>
         <sz val="10"/>
       </rPr>
-      <t>LA15 Auslan</t>
+      <t>LA7 Auslan</t>
     </r>
     <r>
       <rPr>
@@ -805,7 +1562,7 @@
         <color rgb="FFD4538A"/>
         <sz val="10"/>
       </rPr>
-      <t>LA22 Performing Arts</t>
+      <t>LA24 Performing Arts</t>
     </r>
     <r>
       <rPr>
@@ -822,7 +1579,7 @@
         <color rgb="FFD4538A"/>
         <sz val="10"/>
       </rPr>
-      <t>LA20 Auslan</t>
+      <t>LA22 Auslan</t>
     </r>
     <r>
       <rPr>
@@ -830,6 +1587,28 @@
         <sz val="9"/>
       </rPr>
       <t xml:space="preserve">  Cheryl Peak</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF1F8A82"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA21 STEM</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF1F8A82"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Lis Lowndes</t>
     </r>
     <r>
       <rPr>
@@ -844,7 +1623,7 @@
         <color rgb="FF4A90D9"/>
         <sz val="10"/>
       </rPr>
-      <t>LA18 Health</t>
+      <t>LA9 Health</t>
     </r>
     <r>
       <rPr>
@@ -853,20 +1632,26 @@
       </rPr>
       <t xml:space="preserve">  Aaron Bell</t>
     </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Recess
+1:20-1:35</t>
+  </si>
+  <si>
+    <t>Recess (1:20-1:35)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P6
+1:35-2:35</t>
+  </si>
+  <si>
     <r>
       <rPr>
         <b/>
         <color rgb="FF1F8A82"/>
         <sz val="10"/>
       </rPr>
-      <t>LA15 STEM</t>
+      <t>LA22 STEM</t>
     </r>
     <r>
       <rPr>
@@ -875,26 +1660,20 @@
       </rPr>
       <t xml:space="preserve">  Lis Lowndes</t>
     </r>
-  </si>
-  <si>
-    <t xml:space="preserve">Lunch
-11:10-11:50</t>
-  </si>
-  <si>
-    <t>Lunch (11:10-11:50)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P4
-11:50-12:35</t>
-  </si>
-  <si>
+    <r>
+      <rPr>
+        <sz val="6"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
     <r>
       <rPr>
         <b/>
         <color rgb="FFD98A3D"/>
         <sz val="10"/>
       </rPr>
-      <t>LA18 Visual Art</t>
+      <t>LA17 Visual Art</t>
     </r>
     <r>
       <rPr>
@@ -911,7 +1690,7 @@
         <color rgb="FF29A39A"/>
         <sz val="10"/>
       </rPr>
-      <t>LA9 STEM</t>
+      <t>LA6 STEM</t>
     </r>
     <r>
       <rPr>
@@ -919,6 +1698,28 @@
         <sz val="9"/>
       </rPr>
       <t xml:space="preserve">  Chantel Uhe</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF1F8A82"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA18 STEM</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF1F8A82"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Lis Lowndes</t>
     </r>
     <r>
       <rPr>
@@ -933,7 +1734,7 @@
         <color rgb="FFD4538A"/>
         <sz val="10"/>
       </rPr>
-      <t>LA17 Performing Arts</t>
+      <t>LA14 Performing Arts</t>
     </r>
     <r>
       <rPr>
@@ -941,6 +1742,67 @@
         <sz val="9"/>
       </rPr>
       <t xml:space="preserve">  Cheryl Peak</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FFD98A3D"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA20 Visual Art</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FFD98A3D"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Natalie Carter</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF29A39A"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA7 STEM</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF29A39A"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Chantel Uhe</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF7E57C2"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA21 Auslan</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF7E57C2"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Rachel Walker</t>
     </r>
     <r>
       <rPr>
@@ -955,7 +1817,7 @@
         <color rgb="FF1F8A82"/>
         <sz val="10"/>
       </rPr>
-      <t>LA23 STEM</t>
+      <t>LA23 Health</t>
     </r>
     <r>
       <rPr>
@@ -963,6 +1825,28 @@
         <sz val="9"/>
       </rPr>
       <t xml:space="preserve">  Lis Lowndes</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FFD4538A"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA15 Performing Arts</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FFD4538A"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Cheryl Peak</t>
     </r>
     <r>
       <rPr>
@@ -977,7 +1861,7 @@
         <color rgb="FFD98A3D"/>
         <sz val="10"/>
       </rPr>
-      <t>LA7 Visual Art</t>
+      <t>LA9 Visual Art</t>
     </r>
     <r>
       <rPr>
@@ -991,17 +1875,17 @@
     <r>
       <rPr>
         <b/>
-        <color rgb="FF29A39A"/>
+        <color rgb="FF1F8A82"/>
         <sz val="10"/>
       </rPr>
-      <t>LA16 STEM</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FF29A39A"/>
+      <t>LA22 PE</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF1F8A82"/>
         <sz val="9"/>
       </rPr>
-      <t xml:space="preserve">  Chantel Uhe</t>
+      <t xml:space="preserve">  Lis Lowndes</t>
     </r>
     <r>
       <rPr>
@@ -1013,17 +1897,61 @@
     <r>
       <rPr>
         <b/>
-        <color rgb="FFD98A3D"/>
+        <color rgb="FF4A90D9"/>
         <sz val="10"/>
       </rPr>
-      <t>LA22 Visual Art</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FFD98A3D"/>
+      <t>LA23 PE</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF4A90D9"/>
         <sz val="9"/>
       </rPr>
-      <t xml:space="preserve">  Natalie Carter</t>
+      <t xml:space="preserve">  Aaron Bell</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF6AA9E0"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA24 PE</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF6AA9E0"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Jake Pevitt</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="6"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF7E57C2"/>
+        <sz val="10"/>
+      </rPr>
+      <t>LA16 Auslan</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF7E57C2"/>
+        <sz val="9"/>
+      </rPr>
+      <t xml:space="preserve">  Rachel Walker</t>
     </r>
     <r>
       <rPr>
@@ -1038,7 +1966,7 @@
         <color rgb="FFD4538A"/>
         <sz val="10"/>
       </rPr>
-      <t>LA23 Performing Arts</t>
+      <t>LA8 Performing Arts</t>
     </r>
     <r>
       <rPr>
@@ -1047,66 +1975,22 @@
       </rPr>
       <t xml:space="preserve">  Cheryl Peak</t>
     </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
+  </si>
+  <si>
     <r>
       <rPr>
         <b/>
-        <color rgb="FF7E57C2"/>
+        <color rgb="FFD4538A"/>
         <sz val="10"/>
       </rPr>
-      <t>LA24 Auslan</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FF7E57C2"/>
+      <t>LA19 Auslan</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FFD4538A"/>
         <sz val="9"/>
       </rPr>
-      <t xml:space="preserve">  Rachel Walker</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF1F8A82"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA19 STEM</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FF1F8A82"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Lis Lowndes</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF1F8A82"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA14 PE</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FF1F8A82"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Lis Lowndes</t>
+      <t xml:space="preserve">  Cheryl Peak</t>
     </r>
     <r>
       <rPr>
@@ -1121,7 +2005,7 @@
         <color rgb="FF4A90D9"/>
         <sz val="10"/>
       </rPr>
-      <t>LA15 PE</t>
+      <t>LA24 Health</t>
     </r>
     <r>
       <rPr>
@@ -1130,912 +2014,6 @@
       </rPr>
       <t xml:space="preserve">  Aaron Bell</t>
     </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF6AA9E0"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA21 PE</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FF6AA9E0"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Jake Pevitt</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF7E57C2"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA17 Auslan</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FF7E57C2"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Rachel Walker</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FFD4538A"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA19 Performing Arts</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FFD4538A"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Cheryl Peak</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FFD4538A"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA23 Auslan</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FFD4538A"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Cheryl Peak</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF4A90D9"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA22 Health</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FF4A90D9"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Aaron Bell</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF1F8A82"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA21 STEM</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FF1F8A82"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Lis Lowndes</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">P5
-12:35-1:20</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF1F8A82"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA22 STEM</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FF1F8A82"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Lis Lowndes</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FFD98A3D"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA24 Visual Art</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FFD98A3D"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Natalie Carter</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF29A39A"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA6 STEM</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FF29A39A"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Chantel Uhe</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FFD4538A"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA7 Performing Arts</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FFD4538A"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Cheryl Peak</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF1F8A82"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA18 STEM</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FF1F8A82"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Lis Lowndes</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FFD98A3D"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA16 Visual Art</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FFD98A3D"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Natalie Carter</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF29A39A"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA7 STEM</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FF29A39A"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Chantel Uhe</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF7E57C2"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA9 Auslan</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FF7E57C2"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Rachel Walker</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF1F8A82"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA19 STEM</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FF1F8A82"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Lis Lowndes</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FFD98A3D"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA8 Visual Art</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FFD98A3D"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Natalie Carter</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FFD4538A"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA18 Performing Arts</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FFD4538A"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Cheryl Peak</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF1F8A82"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA18 PE</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FF1F8A82"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Lis Lowndes</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF4A90D9"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA19 PE</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FF4A90D9"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Aaron Bell</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF6AA9E0"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA20 PE</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FF6AA9E0"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Jake Pevitt</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF7E57C2"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA7 Auslan</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FF7E57C2"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Rachel Walker</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FFD4538A"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA24 Performing Arts</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FFD4538A"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Cheryl Peak</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FFD4538A"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA22 Auslan</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FFD4538A"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Cheryl Peak</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF1F8A82"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA21 STEM</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FF1F8A82"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Lis Lowndes</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF4A90D9"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA9 Health</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FF4A90D9"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Aaron Bell</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">Recess
-1:20-1:35</t>
-  </si>
-  <si>
-    <t>Recess (1:20-1:35)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P6
-1:35-2:35</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF1F8A82"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA22 STEM</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FF1F8A82"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Lis Lowndes</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FFD98A3D"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA17 Visual Art</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FFD98A3D"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Natalie Carter</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF29A39A"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA6 STEM</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FF29A39A"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Chantel Uhe</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF1F8A82"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA18 STEM</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FF1F8A82"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Lis Lowndes</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FFD4538A"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA14 Performing Arts</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FFD4538A"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Cheryl Peak</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FFD98A3D"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA20 Visual Art</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FFD98A3D"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Natalie Carter</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF29A39A"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA7 STEM</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FF29A39A"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Chantel Uhe</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF7E57C2"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA21 Auslan</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FF7E57C2"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Rachel Walker</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF1F8A82"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA23 Health</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FF1F8A82"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Lis Lowndes</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FFD4538A"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA15 Performing Arts</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FFD4538A"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Cheryl Peak</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FFD98A3D"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA9 Visual Art</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FFD98A3D"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Natalie Carter</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF1F8A82"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA22 PE</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FF1F8A82"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Lis Lowndes</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF4A90D9"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA23 PE</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FF4A90D9"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Aaron Bell</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF6AA9E0"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA24 PE</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FF6AA9E0"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Jake Pevitt</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF7E57C2"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA16 Auslan</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FF7E57C2"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Rachel Walker</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FFD4538A"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA8 Performing Arts</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FFD4538A"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Cheryl Peak</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FFD4538A"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA19 Auslan</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FFD4538A"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Cheryl Peak</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF4A90D9"/>
-        <sz val="10"/>
-      </rPr>
-      <t>LA24 Health</t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FF4A90D9"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">  Aaron Bell</t>
-    </r>
   </si>
   <si>
     <t>Mon · whole school (specialist in colour, otherwise classroom teacher)</t>
@@ -2152,6 +2130,10 @@
     <t>P1 8:55-9:40</t>
   </si>
   <si>
+    <t xml:space="preserve">STEM
+Lis Lowndes</t>
+  </si>
+  <si>
     <t xml:space="preserve">Visual Art
 Natalie Carter</t>
   </si>
@@ -2159,10 +2141,6 @@
     <t>P2 9:40-10:25</t>
   </si>
   <si>
-    <t xml:space="preserve">STEM
-Lis Lowndes</t>
-  </si>
-  <si>
     <t>P3 10:25-11:10</t>
   </si>
   <si>
@@ -2491,6 +2469,10 @@
     <t>Lis Lowndes  ·  specialist (1.0; works Mon/Tue/Wed/Thu/Fri)</t>
   </si>
   <si>
+    <t xml:space="preserve">LA20 (2)
+STEM</t>
+  </si>
+  <si>
     <t xml:space="preserve">LA24 (1)
 STEM</t>
   </si>
@@ -2499,10 +2481,6 @@
 STEM/PE team</t>
   </si>
   <si>
-    <t xml:space="preserve">LA20 (2)
-STEM</t>
-  </si>
-  <si>
     <t xml:space="preserve">LA14 (3/4)
 STEM</t>
   </si>
@@ -2511,6 +2489,10 @@
 PE</t>
   </si>
   <si>
+    <t xml:space="preserve">Cover LA1
+(Luca)</t>
+  </si>
+  <si>
     <t xml:space="preserve">LA15 (3)
 STEM</t>
   </si>
@@ -2555,10 +2537,6 @@
 PE</t>
   </si>
   <si>
-    <t xml:space="preserve">Cover LA1
-(Luca)</t>
-  </si>
-  <si>
     <t>Natalie Carter  ·  specialist (0.6; works Mon/Tue/Wed)</t>
   </si>
   <si>
@@ -3096,7 +3074,7 @@
     <t>4. Monday P0 and P1 vacancy</t>
   </si>
   <si>
-    <t>Monday P0 specialist lessons: 0. Monday P1 specialist lessons: 1. Clear of all specialist activity: FAIL.</t>
+    <t>Monday P0 specialist lessons: 0. Monday P1 specialist lessons: 2. Clear of all specialist activity: FAIL.</t>
   </si>
   <si>
     <t>5. DOTT equity</t>
@@ -3300,7 +3278,7 @@
     <t>| LA14 | 0 | 2 | 2 | 2 | 0 | 2 |</t>
   </si>
   <si>
-    <t>| LA15 | 0 | 0 | 2 | 2 | 2 | 2 |</t>
+    <t>| LA15 | 2 | 0 | 2 | 2 | 0 | 2 |</t>
   </si>
   <si>
     <t>| LA16 | 0 | 2 | 2 | 2 | 0 | 2 |</t>
@@ -3363,7 +3341,7 @@
     <t>STEM (rule 5): every STEM block is two back-to-back periods (consecutive period numbers, same day): PASS.</t>
   </si>
   <si>
-    <t>Specialist teaching by period (rule 7 aims to keep mornings lighter for literacy): P1:7  P2:16  P3:18  P4:18  P5:19  P6:18. Note Thursday PE necessarily fills some morning slots; the rest of the week is pushed later where the other hard rules allow.</t>
+    <t>Specialist teaching by period (rule 7 aims to keep mornings lighter for literacy): P1:8  P2:15  P3:17  P4:19  P5:19  P6:18. Note Thursday PE necessarily fills some morning slots; the rest of the week is pushed later where the other hard rules allow.</t>
   </si>
   <si>
     <t>10. Pre-Primary &amp; Kindy DOTT ledger</t>
@@ -3384,7 +3362,7 @@
     <t>| Katie Digney | PP | LA1 | 0.8 | 256m | 265m | +9m |</t>
   </si>
   <si>
-    <t>| Nikki Luca | PP | LA1 | 0.4 | 128m | 105m | -23m |</t>
+    <t>| Nikki Luca | PP | LA1 | 0.4 | 128m | 135m | +7m |</t>
   </si>
   <si>
     <t>| Kelly Duggan | Kindy | LA4 | 0.8 | 256m | 260m | +4m |</t>
@@ -3496,12 +3474,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFD98A3D"/>
+        <fgColor rgb="FF1F8A82"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF1F8A82"/>
+        <fgColor rgb="FFD98A3D"/>
       </patternFill>
     </fill>
     <fill>
@@ -4346,8 +4324,8 @@
       <c r="K4" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="L4" s="9" t="s">
-        <v>75</v>
+      <c r="L4" s="10" t="s">
+        <v>81</v>
       </c>
       <c r="M4" s="9" t="s">
         <v>76</v>
@@ -4355,8 +4333,8 @@
       <c r="N4" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="O4" s="10" t="s">
-        <v>81</v>
+      <c r="O4" s="11" t="s">
+        <v>82</v>
       </c>
       <c r="P4" s="9" t="s">
         <v>79</v>
@@ -4364,10 +4342,10 @@
     </row>
     <row r="5" ht="32" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="B5" s="11" t="s">
         <v>82</v>
-      </c>
-      <c r="B5" s="10" t="s">
-        <v>81</v>
       </c>
       <c r="C5" s="9" t="s">
         <v>66</v>
@@ -4396,8 +4374,8 @@
       <c r="K5" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="L5" s="11" t="s">
-        <v>83</v>
+      <c r="L5" s="10" t="s">
+        <v>81</v>
       </c>
       <c r="M5" s="9" t="s">
         <v>76</v>
@@ -4431,8 +4409,8 @@
       <c r="F6" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="G6" s="9" t="s">
-        <v>70</v>
+      <c r="G6" s="10" t="s">
+        <v>81</v>
       </c>
       <c r="H6" s="9" t="s">
         <v>71</v>
@@ -4446,8 +4424,8 @@
       <c r="K6" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="L6" s="11" t="s">
-        <v>83</v>
+      <c r="L6" s="9" t="s">
+        <v>75</v>
       </c>
       <c r="M6" s="9" t="s">
         <v>76</v>
@@ -4503,8 +4481,8 @@
       <c r="F8" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="G8" s="9" t="s">
-        <v>70</v>
+      <c r="G8" s="10" t="s">
+        <v>81</v>
       </c>
       <c r="H8" s="9" t="s">
         <v>71</v>
@@ -4512,8 +4490,8 @@
       <c r="I8" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="J8" s="10" t="s">
-        <v>81</v>
+      <c r="J8" s="11" t="s">
+        <v>82</v>
       </c>
       <c r="K8" s="9" t="s">
         <v>74</v>
@@ -4574,14 +4552,14 @@
       <c r="M9" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="N9" s="11" t="s">
-        <v>83</v>
+      <c r="N9" s="10" t="s">
+        <v>81</v>
       </c>
       <c r="O9" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="P9" s="10" t="s">
-        <v>81</v>
+      <c r="P9" s="11" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="10" ht="14" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
@@ -4631,8 +4609,8 @@
       <c r="H11" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="I11" s="10" t="s">
-        <v>81</v>
+      <c r="I11" s="11" t="s">
+        <v>82</v>
       </c>
       <c r="J11" s="9" t="s">
         <v>73</v>
@@ -4646,8 +4624,8 @@
       <c r="M11" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="N11" s="11" t="s">
-        <v>83</v>
+      <c r="N11" s="10" t="s">
+        <v>81</v>
       </c>
       <c r="O11" s="9" t="s">
         <v>78</v>
@@ -4822,13 +4800,13 @@
       <c r="O16" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="P16" s="11" t="s">
-        <v>83</v>
+      <c r="P16" s="10" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="17" ht="32" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B17" s="9" t="s">
         <v>65</v>
@@ -4857,8 +4835,8 @@
       <c r="J17" s="9" t="s">
         <v>73</v>
       </c>
-      <c r="K17" s="10" t="s">
-        <v>81</v>
+      <c r="K17" s="11" t="s">
+        <v>82</v>
       </c>
       <c r="L17" s="13" t="s">
         <v>92</v>
@@ -4872,8 +4850,8 @@
       <c r="O17" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="P17" s="11" t="s">
-        <v>83</v>
+      <c r="P17" s="10" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="18" ht="32" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
@@ -4892,8 +4870,8 @@
       <c r="E18" s="12" t="s">
         <v>91</v>
       </c>
-      <c r="F18" s="10" t="s">
-        <v>81</v>
+      <c r="F18" s="11" t="s">
+        <v>82</v>
       </c>
       <c r="G18" s="9" t="s">
         <v>70</v>
@@ -4919,8 +4897,8 @@
       <c r="N18" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="O18" s="11" t="s">
-        <v>83</v>
+      <c r="O18" s="10" t="s">
+        <v>81</v>
       </c>
       <c r="P18" s="9" t="s">
         <v>79</v>
@@ -4955,8 +4933,8 @@
       <c r="B20" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="C20" s="10" t="s">
-        <v>81</v>
+      <c r="C20" s="11" t="s">
+        <v>82</v>
       </c>
       <c r="D20" s="9" t="s">
         <v>67</v>
@@ -4991,8 +4969,8 @@
       <c r="N20" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="O20" s="11" t="s">
-        <v>83</v>
+      <c r="O20" s="10" t="s">
+        <v>81</v>
       </c>
       <c r="P20" s="9" t="s">
         <v>79</v>
@@ -5020,14 +4998,14 @@
       <c r="G21" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="H21" s="10" t="s">
-        <v>81</v>
+      <c r="H21" s="11" t="s">
+        <v>82</v>
       </c>
       <c r="I21" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="J21" s="11" t="s">
-        <v>83</v>
+      <c r="J21" s="10" t="s">
+        <v>81</v>
       </c>
       <c r="K21" s="9" t="s">
         <v>74</v>
@@ -5098,14 +5076,14 @@
       <c r="I23" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="J23" s="11" t="s">
-        <v>83</v>
+      <c r="J23" s="10" t="s">
+        <v>81</v>
       </c>
       <c r="K23" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="L23" s="10" t="s">
-        <v>81</v>
+      <c r="L23" s="11" t="s">
+        <v>82</v>
       </c>
       <c r="M23" s="9" t="s">
         <v>76</v>
@@ -5277,8 +5255,8 @@
       <c r="L28" s="9" t="s">
         <v>75</v>
       </c>
-      <c r="M28" s="10" t="s">
-        <v>81</v>
+      <c r="M28" s="11" t="s">
+        <v>82</v>
       </c>
       <c r="N28" s="9" t="s">
         <v>77</v>
@@ -5292,7 +5270,7 @@
     </row>
     <row r="29" ht="32" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A29" s="8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B29" s="9" t="s">
         <v>65</v>
@@ -5306,8 +5284,8 @@
       <c r="E29" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="F29" s="11" t="s">
-        <v>83</v>
+      <c r="F29" s="10" t="s">
+        <v>81</v>
       </c>
       <c r="G29" s="9" t="s">
         <v>70</v>
@@ -5356,11 +5334,11 @@
       <c r="E30" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="F30" s="11" t="s">
-        <v>83</v>
-      </c>
-      <c r="G30" s="10" t="s">
+      <c r="F30" s="10" t="s">
         <v>81</v>
+      </c>
+      <c r="G30" s="11" t="s">
+        <v>82</v>
       </c>
       <c r="H30" s="12" t="s">
         <v>91</v>
@@ -5443,8 +5421,8 @@
       <c r="J32" s="9" t="s">
         <v>73</v>
       </c>
-      <c r="K32" s="11" t="s">
-        <v>83</v>
+      <c r="K32" s="10" t="s">
+        <v>81</v>
       </c>
       <c r="L32" s="9" t="s">
         <v>75</v>
@@ -5452,8 +5430,8 @@
       <c r="M32" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="N32" s="10" t="s">
-        <v>81</v>
+      <c r="N32" s="11" t="s">
+        <v>82</v>
       </c>
       <c r="O32" s="13" t="s">
         <v>92</v>
@@ -5472,8 +5450,8 @@
       <c r="C33" s="12" t="s">
         <v>91</v>
       </c>
-      <c r="D33" s="10" t="s">
-        <v>81</v>
+      <c r="D33" s="11" t="s">
+        <v>82</v>
       </c>
       <c r="E33" s="14" t="s">
         <v>94</v>
@@ -5493,8 +5471,8 @@
       <c r="J33" s="13" t="s">
         <v>92</v>
       </c>
-      <c r="K33" s="11" t="s">
-        <v>83</v>
+      <c r="K33" s="10" t="s">
+        <v>81</v>
       </c>
       <c r="L33" s="9" t="s">
         <v>75</v>
@@ -5547,8 +5525,8 @@
       <c r="D35" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="E35" s="10" t="s">
-        <v>81</v>
+      <c r="E35" s="11" t="s">
+        <v>82</v>
       </c>
       <c r="F35" s="9" t="s">
         <v>69</v>
@@ -5577,7 +5555,7 @@
       <c r="N35" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="O35" s="11" t="s">
+      <c r="O35" s="10" t="s">
         <v>95</v>
       </c>
       <c r="P35" s="9" t="s">
@@ -5756,9 +5734,9 @@
     </row>
     <row r="41" ht="32" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A41" s="8" t="s">
-        <v>82</v>
-      </c>
-      <c r="B41" s="11" t="s">
+        <v>83</v>
+      </c>
+      <c r="B41" s="10" t="s">
         <v>97</v>
       </c>
       <c r="C41" s="9" t="s">
@@ -5811,7 +5789,7 @@
       <c r="B42" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="C42" s="11" t="s">
+      <c r="C42" s="10" t="s">
         <v>97</v>
       </c>
       <c r="D42" s="9" t="s">
@@ -5892,7 +5870,7 @@
       <c r="E44" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="F44" s="11" t="s">
+      <c r="F44" s="10" t="s">
         <v>97</v>
       </c>
       <c r="G44" s="15" t="s">
@@ -5954,7 +5932,7 @@
       <c r="I45" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="J45" s="11" t="s">
+      <c r="J45" s="10" t="s">
         <v>97</v>
       </c>
       <c r="K45" s="15" t="s">
@@ -6038,7 +6016,7 @@
       <c r="M47" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="N47" s="11" t="s">
+      <c r="N47" s="10" t="s">
         <v>97</v>
       </c>
       <c r="O47" s="15" t="s">
@@ -6220,7 +6198,7 @@
     </row>
     <row r="53" ht="32" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A53" s="8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B53" s="9" t="s">
         <v>65</v>
@@ -6237,8 +6215,8 @@
       <c r="F53" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="G53" s="11" t="s">
-        <v>83</v>
+      <c r="G53" s="9" t="s">
+        <v>70</v>
       </c>
       <c r="H53" s="9" t="s">
         <v>71</v>
@@ -6287,8 +6265,8 @@
       <c r="F54" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="G54" s="11" t="s">
-        <v>83</v>
+      <c r="G54" s="9" t="s">
+        <v>70</v>
       </c>
       <c r="H54" s="9" t="s">
         <v>71</v>
@@ -6377,8 +6355,8 @@
       <c r="L56" s="9" t="s">
         <v>75</v>
       </c>
-      <c r="M56" s="11" t="s">
-        <v>83</v>
+      <c r="M56" s="10" t="s">
+        <v>81</v>
       </c>
       <c r="N56" s="15" t="s">
         <v>102</v>
@@ -6427,8 +6405,8 @@
       <c r="L57" s="9" t="s">
         <v>75</v>
       </c>
-      <c r="M57" s="11" t="s">
-        <v>83</v>
+      <c r="M57" s="10" t="s">
+        <v>81</v>
       </c>
       <c r="N57" s="13" t="s">
         <v>101</v>
@@ -6616,10 +6594,10 @@
     </row>
     <row r="5" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="B5" s="11" t="s">
         <v>82</v>
-      </c>
-      <c r="B5" s="10" t="s">
-        <v>81</v>
       </c>
       <c r="C5" s="9" t="s">
         <v>65</v>
@@ -6627,7 +6605,7 @@
       <c r="D5" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="E5" s="11" t="s">
+      <c r="E5" s="10" t="s">
         <v>97</v>
       </c>
       <c r="F5" s="9" t="s">
@@ -6810,7 +6788,7 @@
     </row>
     <row r="17" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B17" s="9" t="s">
         <v>66</v>
@@ -6841,7 +6819,7 @@
       <c r="D18" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="E18" s="11" t="s">
+      <c r="E18" s="10" t="s">
         <v>97</v>
       </c>
       <c r="F18" s="9" t="s">
@@ -6867,8 +6845,8 @@
       <c r="B20" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="C20" s="10" t="s">
-        <v>81</v>
+      <c r="C20" s="11" t="s">
+        <v>82</v>
       </c>
       <c r="D20" s="9" t="s">
         <v>66</v>
@@ -7004,7 +6982,7 @@
     </row>
     <row r="29" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B29" s="9" t="s">
         <v>67</v>
@@ -7084,8 +7062,8 @@
       <c r="C33" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="D33" s="10" t="s">
-        <v>81</v>
+      <c r="D33" s="11" t="s">
+        <v>82</v>
       </c>
       <c r="E33" s="9" t="s">
         <v>67</v>
@@ -7198,7 +7176,7 @@
     </row>
     <row r="41" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" s="8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B41" s="9" t="s">
         <v>68</v>
@@ -7310,8 +7288,8 @@
       <c r="C47" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="D47" s="10" t="s">
-        <v>81</v>
+      <c r="D47" s="11" t="s">
+        <v>82</v>
       </c>
       <c r="E47" s="9" t="s">
         <v>68</v>
@@ -7392,7 +7370,7 @@
     </row>
     <row r="53" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" s="8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B53" s="9" t="s">
         <v>69</v>
@@ -7400,8 +7378,8 @@
       <c r="C53" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="D53" s="11" t="s">
-        <v>83</v>
+      <c r="D53" s="10" t="s">
+        <v>81</v>
       </c>
       <c r="E53" s="14" t="s">
         <v>94</v>
@@ -7417,11 +7395,11 @@
       <c r="B54" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="C54" s="10" t="s">
+      <c r="C54" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="D54" s="10" t="s">
         <v>81</v>
-      </c>
-      <c r="D54" s="11" t="s">
-        <v>83</v>
       </c>
       <c r="E54" s="9" t="s">
         <v>69</v>
@@ -7455,7 +7433,7 @@
       <c r="D56" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="E56" s="11" t="s">
+      <c r="E56" s="10" t="s">
         <v>97</v>
       </c>
       <c r="F56" s="9" t="s">
@@ -7586,7 +7564,7 @@
     </row>
     <row r="65" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B65" s="9" t="s">
         <v>70</v>
@@ -7600,28 +7578,28 @@
       <c r="E65" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="F65" s="11" t="s">
-        <v>83</v>
+      <c r="F65" s="9" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="66" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="8" t="s">
         <v>84</v>
       </c>
-      <c r="B66" s="9" t="s">
-        <v>70</v>
+      <c r="B66" s="10" t="s">
+        <v>81</v>
       </c>
       <c r="C66" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="D66" s="10" t="s">
-        <v>81</v>
+      <c r="D66" s="11" t="s">
+        <v>82</v>
       </c>
       <c r="E66" s="14" t="s">
         <v>94</v>
       </c>
-      <c r="F66" s="11" t="s">
-        <v>83</v>
+      <c r="F66" s="9" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="67" ht="14" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -7640,8 +7618,8 @@
       <c r="A68" s="8" t="s">
         <v>86</v>
       </c>
-      <c r="B68" s="9" t="s">
-        <v>70</v>
+      <c r="B68" s="10" t="s">
+        <v>81</v>
       </c>
       <c r="C68" s="9" t="s">
         <v>70</v>
@@ -7780,7 +7758,7 @@
     </row>
     <row r="77" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A77" s="8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B77" s="9" t="s">
         <v>71</v>
@@ -7857,8 +7835,8 @@
       <c r="B81" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="C81" s="10" t="s">
-        <v>81</v>
+      <c r="C81" s="11" t="s">
+        <v>82</v>
       </c>
       <c r="D81" s="9" t="s">
         <v>71</v>
@@ -7974,7 +7952,7 @@
     </row>
     <row r="89" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A89" s="8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B89" s="9" t="s">
         <v>72</v>
@@ -8080,8 +8058,8 @@
       <c r="A95" s="8" t="s">
         <v>89</v>
       </c>
-      <c r="B95" s="10" t="s">
-        <v>81</v>
+      <c r="B95" s="11" t="s">
+        <v>82</v>
       </c>
       <c r="C95" s="9" t="s">
         <v>72</v>
@@ -8168,7 +8146,7 @@
     </row>
     <row r="101" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A101" s="8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B101" s="9" t="s">
         <v>73</v>
@@ -8222,8 +8200,8 @@
       <c r="A104" s="8" t="s">
         <v>86</v>
       </c>
-      <c r="B104" s="10" t="s">
-        <v>81</v>
+      <c r="B104" s="11" t="s">
+        <v>82</v>
       </c>
       <c r="C104" s="9" t="s">
         <v>73</v>
@@ -8245,13 +8223,13 @@
       <c r="B105" s="9" t="s">
         <v>73</v>
       </c>
-      <c r="C105" s="11" t="s">
-        <v>83</v>
+      <c r="C105" s="10" t="s">
+        <v>81</v>
       </c>
       <c r="D105" s="13" t="s">
         <v>92</v>
       </c>
-      <c r="E105" s="11" t="s">
+      <c r="E105" s="10" t="s">
         <v>97</v>
       </c>
       <c r="F105" s="9" t="s">
@@ -8277,8 +8255,8 @@
       <c r="B107" s="9" t="s">
         <v>73</v>
       </c>
-      <c r="C107" s="11" t="s">
-        <v>83</v>
+      <c r="C107" s="10" t="s">
+        <v>81</v>
       </c>
       <c r="D107" s="9" t="s">
         <v>73</v>
@@ -8362,13 +8340,13 @@
     </row>
     <row r="113" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A113" s="8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B113" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="C113" s="10" t="s">
-        <v>81</v>
+      <c r="C113" s="11" t="s">
+        <v>82</v>
       </c>
       <c r="D113" s="9" t="s">
         <v>74</v>
@@ -8422,8 +8400,8 @@
       <c r="C116" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="D116" s="11" t="s">
-        <v>83</v>
+      <c r="D116" s="10" t="s">
+        <v>81</v>
       </c>
       <c r="E116" s="13" t="s">
         <v>92</v>
@@ -8442,8 +8420,8 @@
       <c r="C117" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="D117" s="11" t="s">
-        <v>83</v>
+      <c r="D117" s="10" t="s">
+        <v>81</v>
       </c>
       <c r="E117" s="15" t="s">
         <v>98</v>
@@ -8538,8 +8516,8 @@
       <c r="A124" s="8" t="s">
         <v>80</v>
       </c>
-      <c r="B124" s="9" t="s">
-        <v>75</v>
+      <c r="B124" s="10" t="s">
+        <v>81</v>
       </c>
       <c r="C124" s="9" t="s">
         <v>75</v>
@@ -8556,10 +8534,10 @@
     </row>
     <row r="125" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A125" s="8" t="s">
-        <v>82</v>
-      </c>
-      <c r="B125" s="11" t="s">
         <v>83</v>
+      </c>
+      <c r="B125" s="10" t="s">
+        <v>81</v>
       </c>
       <c r="C125" s="13" t="s">
         <v>92</v>
@@ -8578,8 +8556,8 @@
       <c r="A126" s="8" t="s">
         <v>84</v>
       </c>
-      <c r="B126" s="11" t="s">
-        <v>83</v>
+      <c r="B126" s="9" t="s">
+        <v>75</v>
       </c>
       <c r="C126" s="9" t="s">
         <v>75</v>
@@ -8665,8 +8643,8 @@
       <c r="B131" s="9" t="s">
         <v>75</v>
       </c>
-      <c r="C131" s="10" t="s">
-        <v>81</v>
+      <c r="C131" s="11" t="s">
+        <v>82</v>
       </c>
       <c r="D131" s="9" t="s">
         <v>75</v>
@@ -8738,8 +8716,8 @@
       <c r="C136" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="D136" s="10" t="s">
-        <v>81</v>
+      <c r="D136" s="11" t="s">
+        <v>82</v>
       </c>
       <c r="E136" s="9" t="s">
         <v>76</v>
@@ -8750,7 +8728,7 @@
     </row>
     <row r="137" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A137" s="8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B137" s="9" t="s">
         <v>76</v>
@@ -8816,8 +8794,8 @@
       <c r="E140" s="16" t="s">
         <v>99</v>
       </c>
-      <c r="F140" s="11" t="s">
-        <v>83</v>
+      <c r="F140" s="10" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="141" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -8836,8 +8814,8 @@
       <c r="E141" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="F141" s="11" t="s">
-        <v>83</v>
+      <c r="F141" s="10" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="142" ht="14" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -8944,7 +8922,7 @@
     </row>
     <row r="149" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A149" s="8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B149" s="9" t="s">
         <v>77</v>
@@ -9004,8 +8982,8 @@
       <c r="C152" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="D152" s="10" t="s">
-        <v>81</v>
+      <c r="D152" s="11" t="s">
+        <v>82</v>
       </c>
       <c r="E152" s="9" t="s">
         <v>77</v>
@@ -9018,8 +8996,8 @@
       <c r="A153" s="8" t="s">
         <v>87</v>
       </c>
-      <c r="B153" s="11" t="s">
-        <v>83</v>
+      <c r="B153" s="10" t="s">
+        <v>81</v>
       </c>
       <c r="C153" s="9" t="s">
         <v>77</v>
@@ -9050,8 +9028,8 @@
       <c r="A155" s="8" t="s">
         <v>89</v>
       </c>
-      <c r="B155" s="11" t="s">
-        <v>83</v>
+      <c r="B155" s="10" t="s">
+        <v>81</v>
       </c>
       <c r="C155" s="9" t="s">
         <v>77</v>
@@ -9059,7 +9037,7 @@
       <c r="D155" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="E155" s="11" t="s">
+      <c r="E155" s="10" t="s">
         <v>97</v>
       </c>
       <c r="F155" s="9" t="s">
@@ -9120,8 +9098,8 @@
       <c r="A160" s="8" t="s">
         <v>80</v>
       </c>
-      <c r="B160" s="10" t="s">
-        <v>81</v>
+      <c r="B160" s="11" t="s">
+        <v>82</v>
       </c>
       <c r="C160" s="9" t="s">
         <v>78</v>
@@ -9138,7 +9116,7 @@
     </row>
     <row r="161" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A161" s="8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B161" s="9" t="s">
         <v>78</v>
@@ -9163,8 +9141,8 @@
       <c r="B162" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="C162" s="11" t="s">
-        <v>83</v>
+      <c r="C162" s="10" t="s">
+        <v>81</v>
       </c>
       <c r="D162" s="9" t="s">
         <v>78</v>
@@ -9195,8 +9173,8 @@
       <c r="B164" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="C164" s="11" t="s">
-        <v>83</v>
+      <c r="C164" s="10" t="s">
+        <v>81</v>
       </c>
       <c r="D164" s="13" t="s">
         <v>92</v>
@@ -9250,7 +9228,7 @@
       <c r="C167" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="D167" s="11" t="s">
+      <c r="D167" s="10" t="s">
         <v>95</v>
       </c>
       <c r="E167" s="15" t="s">
@@ -9317,8 +9295,8 @@
       <c r="B172" s="9" t="s">
         <v>79</v>
       </c>
-      <c r="C172" s="11" t="s">
-        <v>83</v>
+      <c r="C172" s="10" t="s">
+        <v>81</v>
       </c>
       <c r="D172" s="9" t="s">
         <v>79</v>
@@ -9332,13 +9310,13 @@
     </row>
     <row r="173" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A173" s="8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B173" s="9" t="s">
         <v>79</v>
       </c>
-      <c r="C173" s="11" t="s">
-        <v>83</v>
+      <c r="C173" s="10" t="s">
+        <v>81</v>
       </c>
       <c r="D173" s="9" t="s">
         <v>79</v>
@@ -9406,8 +9384,8 @@
       <c r="A177" s="8" t="s">
         <v>87</v>
       </c>
-      <c r="B177" s="10" t="s">
-        <v>81</v>
+      <c r="B177" s="11" t="s">
+        <v>82</v>
       </c>
       <c r="C177" s="9" t="s">
         <v>79</v>
@@ -9588,7 +9566,7 @@
     </row>
     <row r="5" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B5" s="17" t="s">
         <v>121</v>
@@ -9782,7 +9760,7 @@
     </row>
     <row r="17" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B17" s="9" t="s">
         <v>126</v>
@@ -9976,7 +9954,7 @@
     </row>
     <row r="29" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B29" s="9" t="s">
         <v>129</v>
@@ -10170,7 +10148,7 @@
     </row>
     <row r="41" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" s="8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B41" s="9" t="s">
         <v>131</v>
@@ -10364,7 +10342,7 @@
     </row>
     <row r="53" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" s="8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B53" s="9" t="s">
         <v>134</v>
@@ -10558,7 +10536,7 @@
     </row>
     <row r="65" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B65" s="9" t="s">
         <v>138</v>
@@ -10572,16 +10550,16 @@
       <c r="E65" s="9" t="s">
         <v>138</v>
       </c>
-      <c r="F65" s="17" t="s">
-        <v>135</v>
+      <c r="F65" s="9" t="s">
+        <v>138</v>
       </c>
     </row>
     <row r="66" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="8" t="s">
         <v>84</v>
       </c>
-      <c r="B66" s="9" t="s">
-        <v>138</v>
+      <c r="B66" s="17" t="s">
+        <v>135</v>
       </c>
       <c r="C66" s="9" t="s">
         <v>138</v>
@@ -10592,8 +10570,8 @@
       <c r="E66" s="17" t="s">
         <v>120</v>
       </c>
-      <c r="F66" s="17" t="s">
-        <v>135</v>
+      <c r="F66" s="9" t="s">
+        <v>138</v>
       </c>
     </row>
     <row r="67" ht="14" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -10612,8 +10590,8 @@
       <c r="A68" s="8" t="s">
         <v>86</v>
       </c>
-      <c r="B68" s="9" t="s">
-        <v>138</v>
+      <c r="B68" s="17" t="s">
+        <v>135</v>
       </c>
       <c r="C68" s="9" t="s">
         <v>138</v>
@@ -10752,7 +10730,7 @@
     </row>
     <row r="77" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A77" s="8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B77" s="9" t="s">
         <v>140</v>
@@ -10946,7 +10924,7 @@
     </row>
     <row r="89" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A89" s="8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B89" s="9" t="s">
         <v>142</v>
@@ -11140,7 +11118,7 @@
     </row>
     <row r="101" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A101" s="8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B101" s="9" t="s">
         <v>144</v>
@@ -11334,7 +11312,7 @@
     </row>
     <row r="113" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A113" s="8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B113" s="9" t="s">
         <v>149</v>
@@ -11510,8 +11488,8 @@
       <c r="A124" s="8" t="s">
         <v>80</v>
       </c>
-      <c r="B124" s="9" t="s">
-        <v>151</v>
+      <c r="B124" s="17" t="s">
+        <v>135</v>
       </c>
       <c r="C124" s="9" t="s">
         <v>151</v>
@@ -11528,7 +11506,7 @@
     </row>
     <row r="125" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A125" s="8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B125" s="17" t="s">
         <v>135</v>
@@ -11550,8 +11528,8 @@
       <c r="A126" s="8" t="s">
         <v>84</v>
       </c>
-      <c r="B126" s="17" t="s">
-        <v>135</v>
+      <c r="B126" s="9" t="s">
+        <v>151</v>
       </c>
       <c r="C126" s="9" t="s">
         <v>151</v>
@@ -11722,7 +11700,7 @@
     </row>
     <row r="137" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A137" s="8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B137" s="9" t="s">
         <v>153</v>
@@ -11916,7 +11894,7 @@
     </row>
     <row r="149" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A149" s="8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B149" s="9" t="s">
         <v>156</v>
@@ -12110,7 +12088,7 @@
     </row>
     <row r="161" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A161" s="8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B161" s="9" t="s">
         <v>160</v>
@@ -12304,7 +12282,7 @@
     </row>
     <row r="173" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A173" s="8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B173" s="9" t="s">
         <v>164</v>
@@ -12498,7 +12476,7 @@
     </row>
     <row r="185" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A185" s="8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B185" s="20" t="s">
         <v>167</v>
@@ -12674,17 +12652,17 @@
       <c r="A196" s="8" t="s">
         <v>80</v>
       </c>
-      <c r="B196" s="21" t="s">
-        <v>168</v>
-      </c>
-      <c r="C196" s="11" t="s">
+      <c r="B196" s="10" t="s">
         <v>177</v>
+      </c>
+      <c r="C196" s="10" t="s">
+        <v>178</v>
       </c>
       <c r="D196" s="21" t="s">
         <v>168</v>
       </c>
       <c r="E196" s="18" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="F196" s="21" t="s">
         <v>168</v>
@@ -12692,21 +12670,21 @@
     </row>
     <row r="197" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A197" s="8" t="s">
-        <v>82</v>
-      </c>
-      <c r="B197" s="11" t="s">
-        <v>179</v>
-      </c>
-      <c r="C197" s="11" t="s">
+        <v>83</v>
+      </c>
+      <c r="B197" s="10" t="s">
         <v>177</v>
       </c>
-      <c r="D197" s="11" t="s">
+      <c r="C197" s="10" t="s">
+        <v>178</v>
+      </c>
+      <c r="D197" s="10" t="s">
         <v>180</v>
       </c>
-      <c r="E197" s="11" t="s">
+      <c r="E197" s="10" t="s">
         <v>181</v>
       </c>
-      <c r="F197" s="11" t="s">
+      <c r="F197" s="22" t="s">
         <v>182</v>
       </c>
     </row>
@@ -12714,19 +12692,19 @@
       <c r="A198" s="8" t="s">
         <v>84</v>
       </c>
-      <c r="B198" s="11" t="s">
-        <v>179</v>
-      </c>
-      <c r="C198" s="11" t="s">
+      <c r="B198" s="10" t="s">
         <v>183</v>
       </c>
-      <c r="D198" s="11" t="s">
+      <c r="C198" s="10" t="s">
+        <v>184</v>
+      </c>
+      <c r="D198" s="10" t="s">
         <v>180</v>
       </c>
-      <c r="E198" s="11" t="s">
-        <v>184</v>
-      </c>
-      <c r="F198" s="11" t="s">
+      <c r="E198" s="10" t="s">
+        <v>185</v>
+      </c>
+      <c r="F198" s="22" t="s">
         <v>182</v>
       </c>
     </row>
@@ -12746,40 +12724,40 @@
       <c r="A200" s="8" t="s">
         <v>86</v>
       </c>
-      <c r="B200" s="21" t="s">
-        <v>168</v>
-      </c>
-      <c r="C200" s="11" t="s">
+      <c r="B200" s="10" t="s">
         <v>183</v>
       </c>
-      <c r="D200" s="11" t="s">
-        <v>185</v>
-      </c>
-      <c r="E200" s="11" t="s">
+      <c r="C200" s="10" t="s">
+        <v>184</v>
+      </c>
+      <c r="D200" s="10" t="s">
         <v>186</v>
       </c>
-      <c r="F200" s="11" t="s">
+      <c r="E200" s="10" t="s">
         <v>187</v>
+      </c>
+      <c r="F200" s="10" t="s">
+        <v>188</v>
       </c>
     </row>
     <row r="201" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A201" s="8" t="s">
         <v>87</v>
       </c>
-      <c r="B201" s="11" t="s">
+      <c r="B201" s="10" t="s">
+        <v>189</v>
+      </c>
+      <c r="C201" s="10" t="s">
+        <v>190</v>
+      </c>
+      <c r="D201" s="10" t="s">
+        <v>186</v>
+      </c>
+      <c r="E201" s="10" t="s">
+        <v>191</v>
+      </c>
+      <c r="F201" s="10" t="s">
         <v>188</v>
-      </c>
-      <c r="C201" s="11" t="s">
-        <v>189</v>
-      </c>
-      <c r="D201" s="11" t="s">
-        <v>185</v>
-      </c>
-      <c r="E201" s="11" t="s">
-        <v>190</v>
-      </c>
-      <c r="F201" s="11" t="s">
-        <v>187</v>
       </c>
     </row>
     <row r="202" ht="14" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -12798,20 +12776,20 @@
       <c r="A203" s="8" t="s">
         <v>89</v>
       </c>
-      <c r="B203" s="11" t="s">
-        <v>188</v>
-      </c>
-      <c r="C203" s="11" t="s">
+      <c r="B203" s="10" t="s">
         <v>189</v>
       </c>
-      <c r="D203" s="11" t="s">
-        <v>191</v>
-      </c>
-      <c r="E203" s="11" t="s">
+      <c r="C203" s="10" t="s">
+        <v>190</v>
+      </c>
+      <c r="D203" s="10" t="s">
         <v>192</v>
       </c>
-      <c r="F203" s="22" t="s">
+      <c r="E203" s="10" t="s">
         <v>193</v>
+      </c>
+      <c r="F203" s="21" t="s">
+        <v>168</v>
       </c>
     </row>
     <row r="205" spans="1:6" x14ac:dyDescent="0.25">
@@ -12868,13 +12846,13 @@
       <c r="A208" s="8" t="s">
         <v>80</v>
       </c>
-      <c r="B208" s="10" t="s">
+      <c r="B208" s="11" t="s">
         <v>195</v>
       </c>
       <c r="C208" s="21" t="s">
         <v>168</v>
       </c>
-      <c r="D208" s="10" t="s">
+      <c r="D208" s="11" t="s">
         <v>196</v>
       </c>
       <c r="E208" s="20" t="s">
@@ -12886,12 +12864,12 @@
     </row>
     <row r="209" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A209" s="8" t="s">
-        <v>82</v>
-      </c>
-      <c r="B209" s="10" t="s">
+        <v>83</v>
+      </c>
+      <c r="B209" s="11" t="s">
         <v>197</v>
       </c>
-      <c r="C209" s="10" t="s">
+      <c r="C209" s="11" t="s">
         <v>198</v>
       </c>
       <c r="D209" s="18" t="s">
@@ -12911,10 +12889,10 @@
       <c r="B210" s="19" t="s">
         <v>200</v>
       </c>
-      <c r="C210" s="10" t="s">
+      <c r="C210" s="11" t="s">
         <v>201</v>
       </c>
-      <c r="D210" s="10" t="s">
+      <c r="D210" s="11" t="s">
         <v>202</v>
       </c>
       <c r="E210" s="20" t="s">
@@ -12940,13 +12918,13 @@
       <c r="A212" s="8" t="s">
         <v>86</v>
       </c>
-      <c r="B212" s="10" t="s">
+      <c r="B212" s="11" t="s">
         <v>203</v>
       </c>
-      <c r="C212" s="10" t="s">
+      <c r="C212" s="11" t="s">
         <v>204</v>
       </c>
-      <c r="D212" s="10" t="s">
+      <c r="D212" s="11" t="s">
         <v>205</v>
       </c>
       <c r="E212" s="20" t="s">
@@ -12960,13 +12938,13 @@
       <c r="A213" s="8" t="s">
         <v>87</v>
       </c>
-      <c r="B213" s="10" t="s">
+      <c r="B213" s="11" t="s">
         <v>206</v>
       </c>
-      <c r="C213" s="10" t="s">
+      <c r="C213" s="11" t="s">
         <v>207</v>
       </c>
-      <c r="D213" s="10" t="s">
+      <c r="D213" s="11" t="s">
         <v>208</v>
       </c>
       <c r="E213" s="20" t="s">
@@ -12992,13 +12970,13 @@
       <c r="A215" s="8" t="s">
         <v>89</v>
       </c>
-      <c r="B215" s="10" t="s">
+      <c r="B215" s="11" t="s">
         <v>209</v>
       </c>
-      <c r="C215" s="10" t="s">
+      <c r="C215" s="11" t="s">
         <v>210</v>
       </c>
-      <c r="D215" s="10" t="s">
+      <c r="D215" s="11" t="s">
         <v>211</v>
       </c>
       <c r="E215" s="20" t="s">
@@ -13080,7 +13058,7 @@
     </row>
     <row r="221" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A221" s="8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B221" s="20" t="s">
         <v>169</v>
@@ -13274,7 +13252,7 @@
     </row>
     <row r="233" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A233" s="8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B233" s="20" t="s">
         <v>169</v>
@@ -13460,7 +13438,7 @@
         <v>169</v>
       </c>
       <c r="E244" s="18" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="F244" s="21" t="s">
         <v>168</v>
@@ -13468,7 +13446,7 @@
     </row>
     <row r="245" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A245" s="8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B245" s="20" t="s">
         <v>169</v>
@@ -13662,7 +13640,7 @@
     </row>
     <row r="257" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A257" s="8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B257" s="20" t="s">
         <v>169</v>
@@ -13949,7 +13927,7 @@
     </row>
     <row r="7" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B7" s="9" t="s">
         <v>264</v>
@@ -14143,7 +14121,7 @@
     </row>
     <row r="19" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B19" s="9" t="s">
         <v>266</v>
@@ -14337,7 +14315,7 @@
     </row>
     <row r="31" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" s="8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B31" s="9" t="s">
         <v>268</v>
@@ -14531,7 +14509,7 @@
     </row>
     <row r="43" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" s="8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B43" s="20" t="s">
         <v>169</v>
@@ -14545,8 +14523,8 @@
       <c r="E43" s="9" t="s">
         <v>268</v>
       </c>
-      <c r="F43" s="9" t="s">
-        <v>268</v>
+      <c r="F43" s="21" t="s">
+        <v>168</v>
       </c>
     </row>
     <row r="44" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -14565,8 +14543,8 @@
       <c r="E44" s="9" t="s">
         <v>268</v>
       </c>
-      <c r="F44" s="9" t="s">
-        <v>268</v>
+      <c r="F44" s="21" t="s">
+        <v>168</v>
       </c>
     </row>
     <row r="45" ht="14" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -14649,8 +14627,8 @@
       <c r="E49" s="9" t="s">
         <v>268</v>
       </c>
-      <c r="F49" s="21" t="s">
-        <v>168</v>
+      <c r="F49" s="9" t="s">
+        <v>268</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
@@ -14725,7 +14703,7 @@
     </row>
     <row r="55" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" s="8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B55" s="9" t="s">
         <v>271</v>
@@ -14919,7 +14897,7 @@
     </row>
     <row r="67" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B67" s="9" t="s">
         <v>274</v>
@@ -15113,7 +15091,7 @@
     </row>
     <row r="79" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A79" s="8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B79" s="20" t="s">
         <v>169</v>
@@ -15307,7 +15285,7 @@
     </row>
     <row r="91" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A91" s="8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B91" s="21" t="s">
         <v>168</v>
@@ -15501,7 +15479,7 @@
     </row>
     <row r="103" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A103" s="8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B103" s="9" t="s">
         <v>283</v>
@@ -15515,8 +15493,8 @@
       <c r="E103" s="9" t="s">
         <v>284</v>
       </c>
-      <c r="F103" s="9" t="s">
-        <v>284</v>
+      <c r="F103" s="22" t="s">
+        <v>285</v>
       </c>
     </row>
     <row r="104" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -15535,8 +15513,8 @@
       <c r="E104" s="9" t="s">
         <v>284</v>
       </c>
-      <c r="F104" s="9" t="s">
-        <v>284</v>
+      <c r="F104" s="22" t="s">
+        <v>285</v>
       </c>
     </row>
     <row r="105" ht="14" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -15619,8 +15597,8 @@
       <c r="E109" s="9" t="s">
         <v>284</v>
       </c>
-      <c r="F109" s="22" t="s">
-        <v>285</v>
+      <c r="F109" s="9" t="s">
+        <v>284</v>
       </c>
     </row>
     <row r="111" spans="1:6" x14ac:dyDescent="0.25">
@@ -15695,7 +15673,7 @@
     </row>
     <row r="115" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A115" s="8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B115" s="9" t="s">
         <v>287</v>
@@ -15889,7 +15867,7 @@
     </row>
     <row r="127" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A127" s="8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B127" s="9" t="s">
         <v>290</v>
@@ -16083,7 +16061,7 @@
     </row>
     <row r="139" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A139" s="8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B139" s="20" t="s">
         <v>293</v>
@@ -16277,7 +16255,7 @@
     </row>
     <row r="151" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A151" s="8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B151" s="9" t="s">
         <v>291</v>
@@ -16471,7 +16449,7 @@
     </row>
     <row r="163" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A163" s="8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B163" s="20" t="s">
         <v>293</v>
@@ -16665,7 +16643,7 @@
     </row>
     <row r="175" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A175" s="8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B175" s="9" t="s">
         <v>288</v>
@@ -16932,7 +16910,7 @@
     </row>
     <row r="7" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B7" s="9" t="s">
         <v>264</v>
@@ -17126,7 +17104,7 @@
     </row>
     <row r="19" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B19" s="9" t="s">
         <v>266</v>
@@ -17320,7 +17298,7 @@
     </row>
     <row r="31" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" s="8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B31" s="9" t="s">
         <v>268</v>
@@ -17514,7 +17492,7 @@
     </row>
     <row r="43" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" s="8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B43" s="20" t="s">
         <v>169</v>
@@ -17528,8 +17506,8 @@
       <c r="E43" s="9" t="s">
         <v>268</v>
       </c>
-      <c r="F43" s="9" t="s">
-        <v>268</v>
+      <c r="F43" s="21" t="s">
+        <v>168</v>
       </c>
     </row>
     <row r="44" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -17548,8 +17526,8 @@
       <c r="E44" s="9" t="s">
         <v>268</v>
       </c>
-      <c r="F44" s="9" t="s">
-        <v>268</v>
+      <c r="F44" s="21" t="s">
+        <v>168</v>
       </c>
     </row>
     <row r="45" ht="14" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -17632,8 +17610,8 @@
       <c r="E49" s="9" t="s">
         <v>268</v>
       </c>
-      <c r="F49" s="21" t="s">
-        <v>168</v>
+      <c r="F49" s="9" t="s">
+        <v>268</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
@@ -17708,7 +17686,7 @@
     </row>
     <row r="55" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" s="8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B55" s="9" t="s">
         <v>271</v>
@@ -17902,7 +17880,7 @@
     </row>
     <row r="67" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B67" s="9" t="s">
         <v>274</v>
@@ -18096,7 +18074,7 @@
     </row>
     <row r="79" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A79" s="8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B79" s="20" t="s">
         <v>169</v>
@@ -18290,7 +18268,7 @@
     </row>
     <row r="91" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A91" s="8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B91" s="21" t="s">
         <v>168</v>
@@ -18484,7 +18462,7 @@
     </row>
     <row r="103" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A103" s="8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B103" s="9" t="s">
         <v>283</v>
@@ -18498,8 +18476,8 @@
       <c r="E103" s="9" t="s">
         <v>284</v>
       </c>
-      <c r="F103" s="9" t="s">
-        <v>284</v>
+      <c r="F103" s="22" t="s">
+        <v>285</v>
       </c>
     </row>
     <row r="104" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -18518,8 +18496,8 @@
       <c r="E104" s="9" t="s">
         <v>284</v>
       </c>
-      <c r="F104" s="9" t="s">
-        <v>284</v>
+      <c r="F104" s="22" t="s">
+        <v>285</v>
       </c>
     </row>
     <row r="105" ht="14" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -18602,8 +18580,8 @@
       <c r="E109" s="9" t="s">
         <v>284</v>
       </c>
-      <c r="F109" s="22" t="s">
-        <v>285</v>
+      <c r="F109" s="9" t="s">
+        <v>284</v>
       </c>
     </row>
     <row r="111" spans="1:6" x14ac:dyDescent="0.25">
@@ -18678,7 +18656,7 @@
     </row>
     <row r="115" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A115" s="8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B115" s="9" t="s">
         <v>287</v>
@@ -18872,7 +18850,7 @@
     </row>
     <row r="127" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A127" s="8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B127" s="9" t="s">
         <v>290</v>
@@ -19066,7 +19044,7 @@
     </row>
     <row r="139" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A139" s="8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B139" s="20" t="s">
         <v>293</v>
@@ -19260,7 +19238,7 @@
     </row>
     <row r="151" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A151" s="8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B151" s="9" t="s">
         <v>291</v>
@@ -19454,7 +19432,7 @@
     </row>
     <row r="163" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A163" s="8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B163" s="20" t="s">
         <v>293</v>
@@ -19648,7 +19626,7 @@
     </row>
     <row r="175" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A175" s="8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B175" s="9" t="s">
         <v>288</v>

</xml_diff>

<commit_message>
Peak leadership: real period at Thu P1; Fri P1 stays DOTT (she runs assembly)
Reverts the Fri P1 stacking - it deleted her actual Events release. Solver
now picks Peak's leadership from Tue-Thu mornings, never Fri P1.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Tapping_S2_Specialist_Timetable.xlsx
+++ b/Tapping_S2_Specialist_Timetable.xlsx
@@ -3103,7 +3103,7 @@
     <t>| Natalie Carter | PBS | Mon P1 | fixed (moved from Mon P3 so LA23 can take P3 - Brad item 5) |</t>
   </si>
   <si>
-    <t>| Cheryl Peak | Events | Fri P1 | leads the Friday assembly (P1 carries no specialist teaching) |</t>
+    <t>| Cheryl Peak | Events | Thu P1 | Peak non-teaching block |</t>
   </si>
   <si>
     <t>| Lincoln Rose | SSTUWA | Fri P2 | LA9 covered by Aaron Bell (Health) · additional 45-min release on top of normal DOTT |</t>
@@ -13093,11 +13093,11 @@
       <c r="D220" s="13" t="s">
         <v>215</v>
       </c>
-      <c r="E220" s="21" t="s">
+      <c r="E220" s="19" t="s">
+        <v>216</v>
+      </c>
+      <c r="F220" s="21" t="s">
         <v>168</v>
-      </c>
-      <c r="F220" s="19" t="s">
-        <v>216</v>
       </c>
     </row>
     <row r="221" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">

</xml_diff>